<commit_message>
update questoes.xlsx: PH02, PH03, PH04, PH05, PH06, PH07, PH08, PH09, PH10
</commit_message>
<xml_diff>
--- a/questoes.xlsx
+++ b/questoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L551"/>
+  <dimension ref="A1:L601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27033,7 +27033,6 @@
           <t>São fotossintetizantes.</t>
         </is>
       </c>
-      <c r="F502" t="inlineStr"/>
       <c r="G502" t="inlineStr">
         <is>
           <t>C</t>
@@ -27054,7 +27053,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K502" t="inlineStr"/>
       <c r="L502" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27088,7 +27086,6 @@
           <t>transformar oxigênio em gás carbônico.</t>
         </is>
       </c>
-      <c r="F503" t="inlineStr"/>
       <c r="G503" t="inlineStr">
         <is>
           <t>C</t>
@@ -27109,7 +27106,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K503" t="inlineStr"/>
       <c r="L503" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27143,7 +27139,6 @@
           <t>temperatura ideal para crescimento.</t>
         </is>
       </c>
-      <c r="F504" t="inlineStr"/>
       <c r="G504" t="inlineStr">
         <is>
           <t>B</t>
@@ -27164,7 +27159,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K504" t="inlineStr"/>
       <c r="L504" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27198,7 +27192,6 @@
           <t>Parasitismo de outros organismos.</t>
         </is>
       </c>
-      <c r="F505" t="inlineStr"/>
       <c r="G505" t="inlineStr">
         <is>
           <t>B</t>
@@ -27219,7 +27212,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K505" t="inlineStr"/>
       <c r="L505" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27253,7 +27245,6 @@
           <t>Paramécios e bactérias.</t>
         </is>
       </c>
-      <c r="F506" t="inlineStr"/>
       <c r="G506" t="inlineStr">
         <is>
           <t>A</t>
@@ -27274,7 +27265,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K506" t="inlineStr"/>
       <c r="L506" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27308,7 +27298,6 @@
           <t>Possui metabolismo e possui nadadeiras.</t>
         </is>
       </c>
-      <c r="F507" t="inlineStr"/>
       <c r="G507" t="inlineStr">
         <is>
           <t>C</t>
@@ -27367,7 +27356,6 @@
           <t>A árvore é autotrófica e não produz seu próprio alimento.</t>
         </is>
       </c>
-      <c r="F508" t="inlineStr"/>
       <c r="G508" t="inlineStr">
         <is>
           <t>A</t>
@@ -27425,7 +27413,6 @@
           <t>Acelular.</t>
         </is>
       </c>
-      <c r="F509" t="inlineStr"/>
       <c r="G509" t="inlineStr">
         <is>
           <t>A</t>
@@ -27446,7 +27433,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K509" t="inlineStr"/>
       <c r="L509" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27482,7 +27468,6 @@
           <t>vírus.</t>
         </is>
       </c>
-      <c r="F510" t="inlineStr"/>
       <c r="G510" t="inlineStr">
         <is>
           <t>D</t>
@@ -27503,7 +27488,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K510" t="inlineStr"/>
       <c r="L510" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27536,7 +27520,6 @@
           <t>capsídeo e núcleo.</t>
         </is>
       </c>
-      <c r="F511" t="inlineStr"/>
       <c r="G511" t="inlineStr">
         <is>
           <t>B</t>
@@ -27557,7 +27540,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K511" t="inlineStr"/>
       <c r="L511" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27590,7 +27572,6 @@
           <t>A diversidade sociocultural do Brasil não está ligada ao território, mas sim à economia global.</t>
         </is>
       </c>
-      <c r="F512" t="inlineStr"/>
       <c r="G512" t="inlineStr">
         <is>
           <t>B</t>
@@ -27611,7 +27592,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K512" t="inlineStr"/>
       <c r="L512" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27645,7 +27625,6 @@
           <t>A noção de território não tem impacto na organização política do Brasil, já que todas as regiões seguem as mesmas políticas públicas.</t>
         </is>
       </c>
-      <c r="F513" t="inlineStr"/>
       <c r="G513" t="inlineStr">
         <is>
           <t>C</t>
@@ -27666,7 +27645,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K513" t="inlineStr"/>
       <c r="L513" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27700,7 +27678,6 @@
           <t>Pela exclusão de influências externas.</t>
         </is>
       </c>
-      <c r="F514" t="inlineStr"/>
       <c r="G514" t="inlineStr">
         <is>
           <t>B</t>
@@ -27721,7 +27698,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K514" t="inlineStr"/>
       <c r="L514" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27755,7 +27731,6 @@
           <t>competição entre o uso agrícola e a preservação ambiental.</t>
         </is>
       </c>
-      <c r="F515" t="inlineStr"/>
       <c r="G515" t="inlineStr">
         <is>
           <t>A</t>
@@ -27776,7 +27751,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K515" t="inlineStr"/>
       <c r="L515" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27810,7 +27784,6 @@
           <t>O Poder Executivo julga casos de violação de leis, o Poder Legislativo executa as políticas públicas, e o Poder Judiciário cria as leis.</t>
         </is>
       </c>
-      <c r="F516" t="inlineStr"/>
       <c r="G516" t="inlineStr">
         <is>
           <t>C</t>
@@ -27831,7 +27804,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K516" t="inlineStr"/>
       <c r="L516" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27872,7 +27844,6 @@
           <t>Estados Unidos, Canadá, África do Sul e Indonésia.</t>
         </is>
       </c>
-      <c r="F517" t="inlineStr"/>
       <c r="G517" t="inlineStr">
         <is>
           <t>C</t>
@@ -27893,7 +27864,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K517" t="inlineStr"/>
       <c r="L517" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -27926,7 +27896,6 @@
           <t>Bolívia e Venezuela.</t>
         </is>
       </c>
-      <c r="F518" t="inlineStr"/>
       <c r="G518" t="inlineStr">
         <is>
           <t>B</t>
@@ -27986,7 +27955,6 @@
           <t>Arroio Chuí.</t>
         </is>
       </c>
-      <c r="F519" t="inlineStr"/>
       <c r="G519" t="inlineStr">
         <is>
           <t>D</t>
@@ -28050,7 +28018,6 @@
           <t>Apenas I, II, e III são verdadeiras.</t>
         </is>
       </c>
-      <c r="F520" t="inlineStr"/>
       <c r="G520" t="inlineStr">
         <is>
           <t>C</t>
@@ -28112,7 +28079,6 @@
           <t>o espaço controlado pelas instituições políticas e militares de um país.</t>
         </is>
       </c>
-      <c r="F521" t="inlineStr"/>
       <c r="G521" t="inlineStr">
         <is>
           <t>D</t>
@@ -28133,7 +28099,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K521" t="inlineStr"/>
       <c r="L521" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28168,7 +28133,6 @@
           <t>A construção de grandes monumentos.</t>
         </is>
       </c>
-      <c r="F522" t="inlineStr"/>
       <c r="G522" t="inlineStr">
         <is>
           <t>B</t>
@@ -28189,7 +28153,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K522" t="inlineStr"/>
       <c r="L522" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28225,7 +28188,6 @@
           <t>impedir o avanço do Império Bizantino no Oriente Médio.</t>
         </is>
       </c>
-      <c r="F523" t="inlineStr"/>
       <c r="G523" t="inlineStr">
         <is>
           <t>C</t>
@@ -28246,7 +28208,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K523" t="inlineStr"/>
       <c r="L523" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28280,7 +28241,6 @@
           <t>Assembleias comerciais.</t>
         </is>
       </c>
-      <c r="F524" t="inlineStr"/>
       <c r="G524" t="inlineStr">
         <is>
           <t>A</t>
@@ -28301,7 +28261,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K524" t="inlineStr"/>
       <c r="L524" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28336,7 +28295,6 @@
           <t>corporações de ofício.</t>
         </is>
       </c>
-      <c r="F525" t="inlineStr"/>
       <c r="G525" t="inlineStr">
         <is>
           <t>D</t>
@@ -28357,7 +28315,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K525" t="inlineStr"/>
       <c r="L525" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28392,7 +28349,6 @@
           <t>descoberta de novas terras.</t>
         </is>
       </c>
-      <c r="F526" t="inlineStr"/>
       <c r="G526" t="inlineStr">
         <is>
           <t>C</t>
@@ -28413,7 +28369,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K526" t="inlineStr"/>
       <c r="L526" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28447,7 +28402,6 @@
           <t>a descoberta de novas vacinas, o que permitiu aos europeus superar doenças fatais como a peste negra.</t>
         </is>
       </c>
-      <c r="F527" t="inlineStr"/>
       <c r="G527" t="inlineStr">
         <is>
           <t>C</t>
@@ -28506,7 +28460,6 @@
           <t>iniciou-se no século XIII e não provocou significativas mudanças no sistema e nas relações feudais vigentes.</t>
         </is>
       </c>
-      <c r="F528" t="inlineStr"/>
       <c r="G528" t="inlineStr">
         <is>
           <t>A</t>
@@ -28570,7 +28523,6 @@
           <t>forma de convencer os fiéis a participarem das expedições.</t>
         </is>
       </c>
-      <c r="F529" t="inlineStr"/>
       <c r="G529" t="inlineStr">
         <is>
           <t>D</t>
@@ -28591,7 +28543,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K529" t="inlineStr"/>
       <c r="L529" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28627,7 +28578,6 @@
           <t>o processo de migração de comerciantes que viviam nos feudos para os burgos.</t>
         </is>
       </c>
-      <c r="F530" t="inlineStr"/>
       <c r="G530" t="inlineStr">
         <is>
           <t>D</t>
@@ -28648,7 +28598,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K530" t="inlineStr"/>
       <c r="L530" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28684,7 +28633,6 @@
           <t>monopólio de determinadas atividades econômicas.</t>
         </is>
       </c>
-      <c r="F531" t="inlineStr"/>
       <c r="G531" t="inlineStr">
         <is>
           <t>D</t>
@@ -28705,7 +28653,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K531" t="inlineStr"/>
       <c r="L531" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28740,7 +28687,6 @@
           <t>Frágil</t>
         </is>
       </c>
-      <c r="F532" t="inlineStr"/>
       <c r="G532" t="inlineStr">
         <is>
           <t>C</t>
@@ -28761,7 +28707,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K532" t="inlineStr"/>
       <c r="L532" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28796,7 +28741,6 @@
           <t>Nomear Poseidon.</t>
         </is>
       </c>
-      <c r="F533" t="inlineStr"/>
       <c r="G533" t="inlineStr">
         <is>
           <t>B</t>
@@ -28817,7 +28761,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K533" t="inlineStr"/>
       <c r="L533" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28857,7 +28800,6 @@
           <t>Rapazinhos.</t>
         </is>
       </c>
-      <c r="F534" t="inlineStr"/>
       <c r="G534" t="inlineStr">
         <is>
           <t>B</t>
@@ -28878,7 +28820,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K534" t="inlineStr"/>
       <c r="L534" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28913,7 +28854,6 @@
           <t>Substantivo comum, concreto.</t>
         </is>
       </c>
-      <c r="F535" t="inlineStr"/>
       <c r="G535" t="inlineStr">
         <is>
           <t>B</t>
@@ -28934,7 +28874,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K535" t="inlineStr"/>
       <c r="L535" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -28970,7 +28909,6 @@
           <t>Brilhantes</t>
         </is>
       </c>
-      <c r="F536" t="inlineStr"/>
       <c r="G536" t="inlineStr">
         <is>
           <t>D</t>
@@ -28991,7 +28929,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K536" t="inlineStr"/>
       <c r="L536" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29041,7 +28978,6 @@
           <t>um substantivo concreto, pois indica o ser denominado.</t>
         </is>
       </c>
-      <c r="F537" t="inlineStr"/>
       <c r="G537" t="inlineStr">
         <is>
           <t>A</t>
@@ -29062,7 +28998,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K537" t="inlineStr"/>
       <c r="L537" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29112,7 +29047,6 @@
           <t>sintagma verbal, por se referir à relação de posse entre a caneca e a água.</t>
         </is>
       </c>
-      <c r="F538" t="inlineStr"/>
       <c r="G538" t="inlineStr">
         <is>
           <t>B</t>
@@ -29133,7 +29067,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K538" t="inlineStr"/>
       <c r="L538" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29169,7 +29102,6 @@
           <t>“interminável”, “prazerosas” e “diferentes”.</t>
         </is>
       </c>
-      <c r="F539" t="inlineStr"/>
       <c r="G539" t="inlineStr">
         <is>
           <t>D</t>
@@ -29190,7 +29122,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K539" t="inlineStr"/>
       <c r="L539" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29228,7 +29159,6 @@
           <t>é parte integral do substantivo e não se refere necessariamente à sua dimensão.</t>
         </is>
       </c>
-      <c r="F540" t="inlineStr"/>
       <c r="G540" t="inlineStr">
         <is>
           <t>D</t>
@@ -29249,7 +29179,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K540" t="inlineStr"/>
       <c r="L540" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29285,7 +29214,6 @@
           <t>de definição e concretização.</t>
         </is>
       </c>
-      <c r="F541" t="inlineStr"/>
       <c r="G541" t="inlineStr">
         <is>
           <t>C</t>
@@ -29306,7 +29234,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K541" t="inlineStr"/>
       <c r="L541" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29340,7 +29267,6 @@
           <t>48</t>
         </is>
       </c>
-      <c r="F542" t="inlineStr"/>
       <c r="G542" t="inlineStr">
         <is>
           <t>B</t>
@@ -29364,7 +29290,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K542" t="inlineStr"/>
       <c r="L542" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29399,7 +29324,6 @@
           <t>Apenas o participante 2, uma vez que a soma deve ser feita da direita para a esquerda.</t>
         </is>
       </c>
-      <c r="F543" t="inlineStr"/>
       <c r="G543" t="inlineStr">
         <is>
           <t>A</t>
@@ -29458,7 +29382,6 @@
           <t>0 e 1</t>
         </is>
       </c>
-      <c r="F544" t="inlineStr"/>
       <c r="G544" t="inlineStr">
         <is>
           <t>A</t>
@@ -29483,7 +29406,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K544" t="inlineStr"/>
       <c r="L544" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29517,7 +29439,6 @@
           <t>Elemento Neutro.</t>
         </is>
       </c>
-      <c r="F545" t="inlineStr"/>
       <c r="G545" t="inlineStr">
         <is>
           <t>C</t>
@@ -29538,7 +29459,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K545" t="inlineStr"/>
       <c r="L545" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29572,7 +29492,6 @@
           <t>60</t>
         </is>
       </c>
-      <c r="F546" t="inlineStr"/>
       <c r="G546" t="inlineStr">
         <is>
           <t>D</t>
@@ -29604,7 +29523,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K546" t="inlineStr"/>
       <c r="L546" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29637,7 +29555,6 @@
           <t>420 figurinhas</t>
         </is>
       </c>
-      <c r="F547" t="inlineStr"/>
       <c r="G547" t="inlineStr">
         <is>
           <t>C</t>
@@ -29658,7 +29575,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K547" t="inlineStr"/>
       <c r="L547" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29691,7 +29607,6 @@
           <t>10</t>
         </is>
       </c>
-      <c r="F548" t="inlineStr"/>
       <c r="G548" t="inlineStr">
         <is>
           <t>A</t>
@@ -29712,7 +29627,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K548" t="inlineStr"/>
       <c r="L548" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29745,7 +29659,6 @@
           <t>100</t>
         </is>
       </c>
-      <c r="F549" t="inlineStr"/>
       <c r="G549" t="inlineStr">
         <is>
           <t>B</t>
@@ -29768,7 +29681,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K549" t="inlineStr"/>
       <c r="L549" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29801,7 +29713,6 @@
           <t>R$ 60,00</t>
         </is>
       </c>
-      <c r="F550" t="inlineStr"/>
       <c r="G550" t="inlineStr">
         <is>
           <t>C</t>
@@ -29823,7 +29734,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K550" t="inlineStr"/>
       <c r="L550" t="inlineStr">
         <is>
           <t>7ano</t>
@@ -29856,7 +29766,6 @@
           <t>4 + (5+2) + 3x1 + 3x7</t>
         </is>
       </c>
-      <c r="F551" t="inlineStr"/>
       <c r="G551" t="inlineStr">
         <is>
           <t>D</t>
@@ -29877,10 +29786,3109 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K551" t="inlineStr"/>
       <c r="L551" t="inlineStr">
         <is>
           <t>7ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>Durante um passeio pelo parque em um dia quente de verão, Pedro percebeu que ao sentar em um banco de madeira, uma leve brisa parecia refrescá-lo. Observou também que, ao se aproximar de um muro, sentia o calor vindo da superfície.
+O que explica a sensação de frescor ao sentir a brisa e o calor ao se aproximar do muro?</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>O ar em movimento (brisa) aquece a superfície do corpo, enquanto o muro libera calor para o ambiente.</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>O ar em movimento (brisa) ajuda a dissipar o calor do corpo, enquanto o muro absorve calor e o libera para o ambiente.</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>O ar em movimento (brisa) retém o calor próximo ao corpo, enquanto o muro resfria o ar ao seu redor.</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>O ar em movimento (brisa) absorve o calor do corpo, enquanto o muro retém calor e o absorve para si.</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>O ar em movimento (brisa) aumenta a temperatura do corpo, enquanto o muro cria uma corrente de ar quente.</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>A brisa aumenta a evaporação do suor e promove a perda de calor do corpo, gerando uma sensação de frescor. O muro, por sua vez, aquece ao absorver calor do sol e libera essa energia para o ambiente, causando a sensação de calor ao se aproximar.</t>
+        </is>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K552" t="inlineStr"/>
+      <c r="L552" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>As correntes oceânicas quentes, como a Corrente do Golfo, transportam calor das regiões equatoriais para latitudes mais altas, enquanto as correntes oceânicas frias, como a Corrente de Humboldt, levam águas mais frias das regiões polares para áreas próximas ao Equador. Esses movimentos influenciam a temperatura e a umidade do ar, afetando o clima de diversas regiões costeiras.
+Disponível em: https://www.todoestudo.com.br/geografia/corrente-de-humboldt.
+A circulação das correntes oceânicas, como a Corrente do Golfo e a Corrente de Humboldt, contribui para:</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>A redução da temperatura das regiões equatoriais, levando águas quentes para os polos.</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>A formação de ventos alísios nas regiões polares, que deslocam o calor para os trópicos.</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>A transferência de calor das regiões tropicais para as temperadas, regulando o clima local.</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>A retenção de calor nos oceanos, mantendo as temperaturas constantes ao longo do ano.</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>A criação de vórtices de ar quente nas zonas polares, aumentando as temperaturas locais.</t>
+        </is>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>As correntes oceânicas são responsáveis por transportar calor das regiões tropicais para as áreas temperadas, influenciando o clima e a temperatura das regiões costeiras ao longo de seu percurso.</t>
+        </is>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K553" t="inlineStr">
+        <is>
+          <t>8a_ph02_cie_02.jpg</t>
+        </is>
+      </c>
+      <c r="L553" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+O vapor d’água proveniente da transpiração das plantas e da evaporação na floresta amazônica, transportado pelas massas de ar, pode ter impacto sobre as chuvas do país, incluindo as regiões Sudeste e Centro-Oeste. Essa é uma das conclusões do projeto ‘Rios voadores’, que vem estudando a importância da floresta amazônica no ciclo hidrológico brasileiro.
+HUCHE, Marcella. Ciência Hoje. Disponível em:  https://cienciahoje.periodicos.capes.gov.br/storage/acervo/ch/ch_260.pdf#page=60 . Acesso em: 21 out. 2024.
+Como as mudanças climáticas globais causadas por ações humanas podem impactar o transporte de vapor d'água na atmosfera e, consequentemente, a circulação das massas de ar e as chuvas nas regiões Sudeste e Centro-Oeste do Brasil?</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Aumento na frequência de massas de ar frias, reduzindo as chuvas.</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Diminuição na intensidade das massas de ar úmidas, reduzindo as chuvas.</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Aumento na frequência de massas de ar secas, aumentando as chuvas.</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>Diminuição na intensidade das massas de ar quentes, aumentando as chuvas.</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>Aumento na frequência de massas de ar úmidas, sem alteração nas chuvas.</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>A diminuição na intensidade das massas de ar úmidas resultaria em menos vapor d'água sendo transportado, o que reduziria as chuvas. Sendo assim, as mudanças climáticas podem alterar os padrões de circulação atmosférica e reduzir a umidade transportada.</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K554" t="inlineStr"/>
+      <c r="L554" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>A circulação atmosférica é um processo dinâmico que envolve a movimentação de massas de ar entre áreas de diferentes pressões. Em regiões de alta pressão, o ar tende a descer e se espalhar horizontalmente, enquanto em regiões de baixa pressão, o ar tende a subir, criando correntes ascendentes. Essas movimentações influenciam diretamente o clima de uma região.
+A circulação atmosférica contribui para a formação de frentes climáticas, pois:</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Mantém o ar estático em regiões de alta e baixa pressão.</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Impede a movimentação de massas de ar entre regiões de diferentes pressões.</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Mantém o ar em movimento horizontal constante em regiões de alta e baixa pressão.</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Move o ar de regiões de alta pressão para baixa pressão, criando correntes ascendentes.</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>Move o ar de regiões de baixa pressão para alta pressão, criando correntes descendentes.</t>
+        </is>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>A circulação atmosférica move o ar de regiões de alta pressão para regiões de baixa pressão. Em regiões de baixa pressão, o ar tende a subir, criando correntes ascendentes que são essenciais para a formação de frentes climáticas.</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K555" t="inlineStr"/>
+      <c r="L555" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>Em regiões costeiras, a presença de grandes corpos d'água, como oceanos, influencia o comportamento do clima local. Durante o dia, a água do mar absorve calor de forma lenta, enquanto a terra aquece mais rapidamente. À noite, a água libera o calor acumulado de forma gradual, fazendo com que a temperatura nas regiões próximas ao mar seja mais amena em comparação com áreas mais afastadas.
+A diferença na absorção e liberação de calor entre a água do mar e a terra é causada principalmente por:</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>A água refletir a maior parte da radiação solar, enquanto a terra a absorve completamente.</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>A água evaporar rapidamente, o que aumenta a temperatura ao redor.</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>A terra liberar calor para a água, que o mantém retido por mais tempo.</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>A água ter uma maior capacidade de armazenar calor do que a terra.</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>A água aquecer e esfriar mais rapidamente que a terra.</t>
+        </is>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>A água possui um alto calor específico, o que significa que ela absorve e libera calor mais lentamente que a terra, resultando em uma moderação da temperatura em regiões costeiras.</t>
+        </is>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K556" t="inlineStr"/>
+      <c r="L556" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>Olhar para o céu durante o dia pode fornecer um indicativo de como estará o tempo daqui algumas horas. As nuvens podem ser um indicativo para a chuva. Nuvens são formadas por:</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>água no estado gasoso, oriunda do espaço.</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>água no estado gasoso, oriunda da atmosfera.</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>água no estado líquido, oriunda do espaço.</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>água do estado líquido, oriunda da condensação da água da atmosfera.</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>água no estado sólido, oriundo do mar, rio ou lago.</t>
+        </is>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>As nuvens são formadas por água no estado liquido, a qual entrou na atmosfera pela vaporização da água presente no planeta (rios, mares, etc.).</t>
+        </is>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K557" t="inlineStr"/>
+      <c r="L557" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>“ O tempo da região sul do Brasil ao longo de 30 anos, sempre foi seco e de temperaturas baixa”.
+A frase acima, quanto ao uso da palavra tempo está:</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>incorreta, pois as condições meteorológicas obtidas ao longo de anos se refere ao clima.</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>incorreta, pois o clima é que é caracterizado pelas condições atmosféricas momentâneas.</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>correta, pois as condições meteorológicas obtidas ao longo de anos se refere ao tempo.</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>correta, pois o clima é que é caracterizado pelas condições atmosféricas momentâneas.</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>correta, pois o tempo se refere aos 30 anos que se passaram.</t>
+        </is>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>A afirmação está incorreta, pois a média das condições atmosféricas mais frequentes em uma região ao longo de um certo intervalo de tempo é chamada de clima. Já o tempo considera as condições atmosféricas momentâneas de uma região.</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K558" t="inlineStr"/>
+      <c r="L558" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>O ciclo da água explica a formação das nuvens e a presença de umidade no ar. As chuvas são formadas pelo vapor de água na atmosfera. Portanto</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>quanto menor a umidade do ar, menor é quantidade vapor de água na atmosfera, logo maior será a probabilidade de chuvas.</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>quanto maior a umidade do ar, maior é quantidade vapor de água na atmosfera, logo maiores serão as chances de ocorrência de chuvas.</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>quanto maior a umidade do ar, maior é quantidade vapor de água na atmosfera, logo menores serão as chances de ocorrência de chuvas.</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>quanto menor a umidade do ar, maior é quantidade vapor de água na atmosfera, logo maior será a probabilidade de chuvas.</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>quanto maior a umidade do ar, menor é quantidade vapor de água na atmosfera, logo maior será a probabilidade de chuvas.</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>A umidade do ar está relacionada com a quantidade de vapor de água na atmosfera. Quanto maior a umidade, maior é a quantidade de vapor de água, logo maior será a probabilidade de chuvas.</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K559" t="inlineStr"/>
+      <c r="L559" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>Disponível em: &lt;http://wwweducacionalnet1.cdn.educacional.com.br/imagens/reportagens/aguas_abril/img_pg7b.jpg&gt;. Acesso em 2 set. 2018.
+A figura mostra a representação de um aparelho que mede a quantidade de chuva de uma região. Ele é chamado de:</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>barômetro.</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>pluviômetro.</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>termômetro.</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>anemômetro.</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>aquametro.</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>O pluviômetro é um cilindro graduado, no qual a água é recolhida e estimada.</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K560" t="inlineStr">
+        <is>
+          <t>8a_ph02_cie_09.jpg</t>
+        </is>
+      </c>
+      <c r="L560" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>Analise a ilustração a seguir.
+Disponível em: &lt;https://cursinhocucafresca.files.wordpress.com/2011/05/dinc3a2mica-climc3a1tica-e-formac3a7c3b5es-vegetais.pdf&gt;. Acesso em: 2 set. 2018.
+O movimento de ar representado indica a formação de uma frente:</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>fria, caracterizada pela chegada de uma massa de ar frio em uma região na qual existe uma massa de ar quente.</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>fria, caracterizada pela chegada de uma massa de ar quente em uma região na qual existe uma massa de ar frio.</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>quente, caracterizada pela chegada de uma massa de ar quente em uma região na qual existe uma massa de ar frio.</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>quente, caracterizada pela chegada de uma massa de ar frio em uma região na qual existe uma massa de ar quente.</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>normal, caracterizada pela chegada de uma massa de ar frio em uma região na qual existe uma massa de ar quente.</t>
+        </is>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>A ilustração mostra a chegada de uma massa de ar frio sobre uma região com uma massa de ar quente, caracterizando a chegada de uma frente fria.</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K561" t="inlineStr">
+        <is>
+          <t>8a_ph02_cie_10.jpg</t>
+        </is>
+      </c>
+      <c r="L561" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>A população humana no planeta apresenta uma diversidade de rotas de dispersão, influenciadas por fatores físicos, naturais e históricos. No continente americano, a colonização, as migrações forçadas e as oportunidades econômicas moldaram os padrões populacionais. Fatores como clima, relevo e recursos naturais também desempenham papéis cruciais na distribuição da população.
+Assinale a alternativa que melhor descreve um fator que contribuiu para a dispersão da população no continente americano.</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Clima frio na América do Sul.</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Presença de grandes desertos no norte da América.</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Disponibilidade de recursos hídricos e terras férteis.</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>Relevo montanhoso na costa oeste da América do Norte.</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>Densidade populacional uniforme em todo o continente.</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>A disponibilidade de recursos hídricos e terras férteis atraiu populações ao longo da história, favorecendo a agricultura e o desenvolvimento de comunidades.</t>
+        </is>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K562" t="inlineStr"/>
+      <c r="L562" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>A América Anglo-Saxônica, composta principalmente pelos Estados Unidos e Canadá, têm sistemas políticos democráticos e uma influência significativa na economia e na cultura global. Além disso, a América Anglo-Saxônica possui vastos recursos naturais, incluindo petróleo, madeira e terras agrícolas.
+Assinale a alternativa que melhor descreve uma característica da América Anglo-Saxônica:</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Alta diversidade cultural e étnica.</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Baixo desenvolvimento econômico.</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Exclusão de influências imigratórias.</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>Predomínio de sistemas autoritários.</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>Riqueza de recursos naturais escassos.</t>
+        </is>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>A América Anglo-Saxônica é conhecida pela alta diversidade cultural e étnica, resultado de longos processos migratórios e coloniais.</t>
+        </is>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K563" t="inlineStr"/>
+      <c r="L563" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>A formação territorial da América Anglo-Saxônica está ligada vários processos históricos, dentre eles a "Marcha para o Oeste" nos Estados Unidos.
+Um aspecto da Marcha para o Oeste nos Estados Unidos foi o(a)</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Estagnação econômica.</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Redução das tensões sociais.</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Aumento da população indígena.</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Conquista de terras para colonização.</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>Integração pacífica com os povos nativos.</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>A Marcha para o Oeste foi marcada pela conquista de terras, visando a colonização e o assentamento, frequentemente em detrimento das populações indígenas.</t>
+        </is>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K564" t="inlineStr"/>
+      <c r="L564" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>A Guerra Civil Americana, ocorrida entre 1861 e 1865, foi um conflito interno nos Estados Unidos. O resultado da guerra teve um impacto significativo na formação territorial e na economia do país.
+Qual das seguintes causas foi um dos principais motivos da Guerra Civil Americana?</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Disputa por territórios com o Canadá.</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Conflito com populações indígenas.</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Questão da escravidão.</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>Expansão para o oeste.</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>Revolução Industrial.</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>A questão da escravidão foi um dos principais motivos da Guerra Civil Americana, gerando divisões profundas entre os estados do norte e do sul.</t>
+        </is>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K565" t="inlineStr"/>
+      <c r="L565" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>A formação territorial do Canadá foi influenciada por diversos eventos históricos, incluindo o Tratado de Paris de 1763. Esse tratado encerrou a Guerra dos Sete Anos e foi crucial para a configuração territorial do Canadá moderno.
+Uma das consequências do Tratado de Paris de 1763 para a formação territorial do Canadá foi a:</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>independência do Canadá da Grã-Bretanha.</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>cessão de territórios franceses para os britânicos.</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>unificação das colônias britânicas na América do Norte.</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>criação da província de Quebec como uma colônia francesa.</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>assinatura de um acordo de livre comércio com os Estados Unidos.</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>O Tratado de Paris de 1763 resultou na cessão de vastos territórios franceses na América do Norte para os britânicos, o que foi crucial para a formação territorial do Canadá moderno.</t>
+        </is>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K566" t="inlineStr"/>
+      <c r="L566" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>Banco de imagens/Arquivo da editora.
+Sistema de ensino PH. EFII9. Caderno 1. Módulo 5.
+A menor ocupação  demográfica na parte norte da América anglo saxônica se deve</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>ao clima frio e polar.</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>ao relevo plano e fértil.</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>a presença de agricultura mecanizada.</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>a rede hidrográfica planáltica.</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>a formação vegetal temperada.</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>A região norte do continente americano é uma área anecúmena - ou seja, de difícil ocupação -, apresentando condições climáticas muito rigorosas. Assim, as características do clima frio e polar dificultam a ocupação dessa área do território anglo-saxônico.</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K567" t="inlineStr">
+        <is>
+          <t>8a_ph02_geo_06.jpg</t>
+        </is>
+      </c>
+      <c r="L567" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+A história dos Estados Unidos da América, hoje conhecida por nós, inicia-se a partir do século XVI, quando exploradores europeus aportaram no lado norte do continente americano. Até então, apenas nativos habitavam no local, a partir dessa conexão com o continente europeu, os Estados Unidos passaram a ser colônia da Inglaterra. Inicialmente estes colonizaram a parte leste do país, o que corresponde ao litoral que é banhado pelo oceano Atlântico. Logo depois a parte central foi colonizada pela França e a parte sudeste e sudoeste pela Espanha.
+[...]
+Disponível em:&lt; https://www.infoescola.com/historia/colonizacao-dos-estados-unidos-da-america/&gt;. Acesso em: 16 mar.2020.
+A relação entre as várias etnias indígenas americanas e o colonizador foi</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>amigável.</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>industrial.</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>comercial.</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>conflituosa.</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>cooperativa.</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>Os colonizadores ingleses não respeitaram as territorialidades indígenas e promoveram o extermínio genocida das populações indígenas através de doenças e do conflito direto pela posse de território.</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K568" t="inlineStr"/>
+      <c r="L568" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Observe o mapa físico de parte da América do Norte:
+Disponível em: &lt; https://www.infoescola.com/wp-content/uploads/2009/08/full-1-e795eccc0c.jpg&gt;. Acesso em: 13 mar 2020.
+O que o aspecto do relevo do oeste da América do Norte revela?</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Áreas com tectonismo inativo.</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Áreas com tectonismo ativo.</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Áreas com baixo aproveitamento hídrico.</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>Áreas com alto aproveitamento hídrico.</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>Área de planícies inundáveis.</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>A costa oeste é reconhecida por cadeias montanhosas entre 1000 e 2000 metros de altitude, tendo origem tectônica.</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K569" t="inlineStr">
+        <is>
+          <t>8a_ph02_geo_08.png</t>
+        </is>
+      </c>
+      <c r="L569" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+O dia 25 de junho de 1876 amanheceu com cheiro e gosto de glória para o general George Armstrong Custer e seus 647 homens da 7ª Cavalaria. Finalmente, a caça aos índios que haviam se rebelado contra o governo dos Estados Unidos tinha chegado ao fim. Ao longo do vale do rio Little Bighorn, no atual estado de Montana, repousava o maior acampamento indígena já visto naquelas bandas.
+[...]
+Só que o general foi cercado.
+[...]
+Custer também foi assassinado. Essa batalha, entretanto, estava longe de ser decisiva. E os sioux estavam bem perto de seu fim como povo. "Essa rebelião indígena tem relação direta com a colonização do Oeste. Até por volta de 1840, os sioux, líderes da revolta, desfrutavam de uma boa convivência com os homens brancos", diz o professor Michael Tate, especialista em nativos americanos, da Universidade de Nebraska, no Estados Unidos.
+ONÇA, Fabiano. SIOUX: VÍTIMAS DO MAIOR GENOCÍDIO DO SÉCULO 19. Disponível em:&lt;https://aventurasnahistoria.uol.com.br/noticias/reportagem/sioux-vitimas-genocidio.phtml&gt;. Acesso em: 13 mar. 2020.
+Os fatos mencionados integram o processo de ocupação do território estadunidense conhecido como:</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Colonização francesa.</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Guerra de secessão.</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Marcha para o Oeste.</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>Destino manifesto.</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>Guerra de independência.</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>Na segunda metade do século XIX, iniciou-se um processo de expansão da costa leste em direção ao oeste dos Estados Unidos, num processo que ficou conhecido como marcha para o oeste, várias ações integraram tal processo e até mesmo uma doutrina religiosa (Destino manifesto).</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K570" t="inlineStr"/>
+      <c r="L570" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+A Corrente do Golfo nunca esteve tão fraca. Segundo pesquisas recentes, a diminuição do volume de água é o menor dos últimos 1.600 anos. Cientistas alertam para a necessidade de reverter a situação para evitar consequências no clima do planeta. As informações foram publicadas pelo jornal The Guardian.
+A corrente do Golfo estaria sendo prejudicada pelo Aquecimento Global. O aumento da temperatura derrete o gelo do Ártico e injeta água doce e fria no Atlântico Norte e isso estaria alterando a circulação da corrente pela diferença de densidade.
+A corrente do Golfo faz parte do sistema chamado Circulação Meridional do Atlântico, um gigantesco fluxo de água no Oceano Atlântico e com impacto no clima. A água quente de áreas tropicais vai em direção ao hemisfério norte, esfria no polo e retorna em direção ao hemisfério sul. Desde 1950, já foi registrado uma redução de 15 % da intensidade desse fluxo.
+Disponível em:&lt; https://noticias.r7.com/tecnologia-e-ciencia/corrente-do-golfo-mais-fraca-compromete-clima-em-todo-planeta18042018&gt;. Acesso em: 17 mar. 2020.
+A corrente do Golfo influencia o clima no EUA na</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Porção oeste.</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Porção leste.</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Porção sul.</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>Porção norte.</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>Porção oeste e sul.</t>
+        </is>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>A Corrente do Golfo é uma corrente quente que influencia o clima europeu, deixando-o com invernos menos rigorosos e também o clima norte-americano, no estado da Flórida, deixando-o mais úmido e quente.</t>
+        </is>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K571" t="inlineStr"/>
+      <c r="L571" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+A Revolução Industrial iniciada na Inglaterra, em meados do século XVIII, com a transição da manufatura para a indústria mecânica, gerando o aumento da produção e a ascensão de novas tecnologias, alterou o modo de vida no planeta.
+POTT, C. M. &amp; ESTRELA, C. C. Histórico ambiental: desastres ambientais e o despertar de um novo pensamento. Disponível em: &lt; http://www.scielo.br/scielo.php?script=sci_arttext&amp;pid=S0103-40142017000100271&gt;. Acesso em: 15 jan. 2020.
+Além das tecnologias ligadas à produção, está entre as consequências do processo conhecido como Revolução Industrial, a(o)</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>invenção do relógio.</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>criação de leis de proteção ao trabalhador.</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>devastação ambiental e a emissão de gases.</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>regulamentação da mão de obra feminina e infantil.</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>expansão dos direitos políticos aos mais pobres.</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>Entre as consequências da Revolução Industrial, está o impacto ambiental causado pelas máquinas, alimentadas por carvão, e que demandavam a exploração de bosques e florestas, além da emissão de gases e fuligem por conta do uso de combustíveis.</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K572" t="inlineStr"/>
+      <c r="L572" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+[...] é a força de trabalho, no seu uso durante a jornada de trabalho pré-determinada, que adianta ao capitalista, na forma de mais-valia, os recursos que colocam a produção em funcionamento. Isso quer dizer que o trabalhador só recebe salários ao fim da jornada de trabalho [...].
+GOMES, Fábio Guedes. Mobilidade do trabalho e controle social: Trabalho e organizações na era neoliberal. Revista de Sociologia e Política v. 17, n. 32. Curitiba: p. 45, 2009. Disponível em: &lt;https://revistas.ufpr.br/rsp/article/view/28213/18727&gt;. Acesso em: 09 jan. 2020.
+O conceito de mais-valia, citado no trecho, designa a(o)</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>acúmulo de capital do burguês.</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>acúmulo de meios de produção pelo burguês.</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>alienação do operário em relação ao salário recebido.</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>tática de aumento do lucro mediante o pagamento de baixas remunerações.</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>diferença entre valor gerado pelo trabalho e pagamento da mão-de-obra.</t>
+        </is>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>Ao pagarem salários mais baixos para seus empregados, os patrões conseguiam aumentar seus lucros. Sendo assim, a mais valia designa a diferença entre o valor produzido pelo trabalho e o pagamento feito pelo patrão aos funcionários.</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K573" t="inlineStr"/>
+      <c r="L573" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+“Os operários não se contentam com dirigir os seus ataques contra as relações burguesas de produção, e dirigem-se contra os próprios instrumentos de produção: destroem as mercadorias estrangeiras que lhes fazem concorrência, quebram as máquinas, incendeiam as fábricas, tentam reconquistar pela força a posição perdida do artesão da Idade Média”.
+COGGIOLA, Osvaldo. O início das organizações dos trabalhadores. Revista Aurora, n. 6. Marília: UNESP, p. 17, 2010. Disponível em: &lt; http://www2.marilia.unesp.br/revistas/index.php/aurora/article/view/1227/1094&gt;. Acesso em: 16 jan. 2020. (Adaptado).
+Os operários descritos pelo autor estão relacionados ao movimento chamado</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>sindical.</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>ludismo.</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>cartismo.</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>revolucionário.</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>resistência operária.</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>O movimento chamado ludismo era caracterizado por ações de trabalhadores que quebravam máquinas, pois as consideravam culpadas pela substituição da mão de obra humana.</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K574" t="inlineStr"/>
+      <c r="L574" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+A Revolução Industrial vai além da ideia de grande desenvolvimento dos mecanismos tecnológicos aplicados à produção, na medida em que: consolidou o capitalismo; aumentou de forma rapidíssima a produtividade do trabalho; originou novos comportamentos sociais, novas formas de acumulação de capital, novos modelos políticos e uma nova visão do mundo; e talvez o mais importante, contribuiu de maneira decisiva para dividir a imensa maioria das sociedades humanas em duas classes sociais opostas e antagônicas [...].
+CAVALCANTE, Zedequias Vieira; SILVA, Mauro Luis Siqueira da. A Importância da Revolução Industrial no Mundo da Tecnologia. In: Anais Eletrônico VII EPCC – Encontro Internacional de Produção Científica Cesumar, p.4. Disponível em: &lt; https://www.unicesumar.edu.br/epcc-2011/wp-content/uploads/sites/86/2016/07/zedequias_vieira_cavalcante2.pdf&gt;. Acesso em: 16 jan. 2020.
+As “duas classes sociais opostas e antagônicas” a qual o texto se refere correspondem a quais segmentos da sociedade?</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Liberais e socialistas.</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Burguesia e operariado.</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Classe média e aristocracia.</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>Republicanos e monarquistas.</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>Progressistas e conservadores.</t>
+        </is>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>Com a Revolução Industrial, os modos de produção e consumo foram alterados drasticamente, acarretando uma nova organização social nas relações de trabalho. Tal processo desencadeou na criação de duas classes sociais elementares para tal organização: os exploradores, representados na burguesia, e os explorados, com o operariado.</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K575" t="inlineStr"/>
+      <c r="L575" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+A Europa da segunda metade do século XVIII foi marcada por profundas mudanças econômicas e sociais. Ideais liberais na França e transformações técnicas e econômicas na Grã-Bretanha deram a “sensação” de ruptura com o passado. A ideia do novo, do progresso, se disseminava pela Europa, que buscava pôr em prática novas invenções que se adequassem ao ritmo do cotidiano alucinante imposto pela nova ordem do trabalho. O tempo tornou-se ainda mais valioso para aqueles que almejavam ganhar dinheiro, de modo que cada minuto deveria ser minuciosamente aproveitado. Nas fábricas, os trabalhadores foram obrigados a seguir o ritmo da máquina a vapor, a qual forneceu um grande impulso ao setor têxtil.
+OLIVEIRA, E. M.. Transformações no Mundo do Trabalho: Da Revolução Industrial aos nossos dias. Caminhos da Geografia (UFU. Online), Uberlândia., v. 11, 2004, p.84-85. (Adaptado).
+A partir do fragmento acima, nota-se como a Revolução Industrial impactou a vida do trabalhador inglês,</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>melhorando o bem-estar do operariado, uma vez que mais riqueza passava a ser gerada e distribuída.</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>alterando o ritmo de trabalho e, por consequência, as relações sociais do operariado que então se formava.</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>levando aos operários ideias revolucionárias advindas dos ideais liberais, o que acarretou diversas revoltas sindicais.</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>mantendo os hábitos e costumes do proletariado, visto que os antigos trabalhadores rurais não conseguiam se adaptar ao ritmo de trabalho fabril.</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>diminuindo a carga de trabalho dos operários, tendo em vista que o progresso técnico visava também a melhoria das condições de vida dos trabalhadores.</t>
+        </is>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>O texto-base descreve algumas das mudanças decorrentes da Revolução Industrial com a chegada de um novo “ritmo do cotidiano alucinante imposto pela nova ordem do trabalho”, fazendo com que os trabalhadores fossem “obrigados a seguir o ritmo da máquina a vapor”. A partir disso, é possível notar como o ritmo do trabalho industrial impactou a vida do operário inglês, mudando não somente sua forma de trabalhar, mas também de se relacionar.</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K576" t="inlineStr"/>
+      <c r="L576" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>A imagem retrata uma cidade industrial típica do século XIX, com uma paisagem marcada pela presença de numerosas chaminés de fábricas. Este cenário é um reflexo das profundas transformações econômicas e sociais ocorridas durante a Revolução Industrial.
+Cidade de Manchester, 1852. Aquarela de William Wyld. Paisagem dominada por chaminés. Royal Collection Trust, Londres, Inglaterra.
+Disponível em: https://acervocmsp.educacao.sp.gov.br/92756/494622.pdf. Acesso em: 17 out. 2024.
+Com base na imagem e no contexto histórico da Revolução Industrial, como esse período contribuiu para o crescimento urbano?</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Aumentando a produção agrícola e migração para áreas rurais.</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Concentrando fábricas em áreas urbanas e com êxodo rural.</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Desenvolvendo novas tecnologias de transporte marítimo.</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>Reduzindo a população urbana devido à mecanização.</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>Estagnando a economia com o declínio das cidades.</t>
+        </is>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>A Revolução Industrial levou à criação de grandes fábricas nas áreas urbanas, atraindo trabalhadores rurais em busca de emprego, o que resultou no crescimento das cidades.</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K577" t="inlineStr">
+        <is>
+          <t>8a_ph02_his_06.png</t>
+        </is>
+      </c>
+      <c r="L577" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+A Revolução Industrial Britânica (1760-1840) testemunhou um grande número de inovações técnicas, como as máquinas a vapor, que resultaram em novas práticas de trabalho, que por sua vez trouxeram muitas mudanças sociais. Mais mulheres e crianças trabalhavam do que antes; pela primeira vez, os habitantes de vilas e cidades superaram os do campo; as pessoas se casavam mais jovens e tinham mais filhos; e a dieta da população melhorou. A mão de obra tornou-se muito menos qualificada do que antes e as novas instalações fabris se transformaram em locais insalubres e perigosos. As cidades sofriam com a poluição, a falta de saneamento e a criminalidade.  
+As Mudanças Sociais na Revolução Industrial Britânica. Disponível em: https://www.worldhistory.org/trans/pt/2-2229/as-mudancas-sociais-na-revolucao-industrial-britan/#google_vignette. Acesso em: 25 out. 2024.
+Como a Revolução Industrial ampliou a divisão entre a burguesia e o proletariado?</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Criando uma classe de proprietários de fábricas ricos em oposição à aristocracia decadente.</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Intensificando a urbanização devido ao uso das terras dos camponeses para a produção de lã.</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>Aumentando a produção e a eficiência nas fábricas sem distribuir os lucros de forma equitativa.</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>Proporcionando oportunidades de emprego estável com remuneração elevada para mais pessoas.</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>Introduzindo novas tecnologias que aumentaram a produtividade e ofereceram mercadorias baratas a todos.</t>
+        </is>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>Revolução Industrial acentuou a divisão entre a burguesia e o proletariado pois a burguesia, proprietária dos meios de produção, detinha fábricas altamente produtivas e eficientes, mas que dependiam dos trabalhadores para funcionarem. Ao não distribuir as riquezas produzidas, as contradições entre burguesia e proletariado se intensificaram.</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K578" t="inlineStr"/>
+      <c r="L578" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+[...] foi um dos desenvolvimentos mais significativos da Revolução Industrial (1760-1840) na Grã-Bretanha. Empregada inicialmente em bombas de drenagem na década de 1690, uma série de inventores aperfeiçoou seus mecanismos, criando equipamentos que se tornaram uma alternativa eficiente e poderosa à energia dos músculos, da água e do vento, com real viabilidade econômica. 
+Disponível em: https://www.worldhistory.org/trans/pt/2-2166/. Acesso em 25 out. 2024.
+Qual invenção foi crucial para o desenvolvimento da Revolução Industrial?</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Telefone</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Telégrafo</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Computador</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>Máquina a vapor</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>Motor de combustão interna</t>
+        </is>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>A máquina a vapor foi crucial para o desenvolvimento da Revolução Industrial, sendo amplamente utilizada nas fábricas e nos transportes.</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K579" t="inlineStr"/>
+      <c r="L579" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+[...] este é reconhecido com a elaboração da Carta do Povo, que exigia o direito de votar e ser votado. Esse movimento direcionou a luta pelo direito ao sufrágio universal, despertando no proletariado o desejo de acabar com a sua impotência política.
+A organização política da classe operária do século XIX. Disponível em: http://www.ubimuseum.ubi.pt/n02/docs/ubimuseum02/ubimuseum02.fernando-araujo-reivan-souza.pdf. Acesso em: 25 out. 2024.
+Qual foi o importante movimento de trabalhadores trabalhado no texto que surgiu com o desenvolvimento da Revolução Industrial?</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Cartismo.</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Sindicalismo.</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>Ludismo.</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>Socialismo.</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>Anarquismo.</t>
+        </is>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>O movimento cartista baseava-se na Carta do Povo, exigindo reformas econômicas e políticas, como a redução da jornada de trabalho e o sufrágio universal, em defesa dos trabalhadores.</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K580" t="inlineStr"/>
+      <c r="L580" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+Fazer bicos para sustentar a família ou complementar a renda não é novidade. Mas a forma como esses bicos ocorrem hoje em dia se tornou tão mediada pela tecnologia que ganhou um termo próprio em inglês: gig economy. A gig economy se refere aos tipos de trabalho em que a pessoa faz tarefas sob demanda, geralmente por meio de uma plataforma, como Uber e iFood. Por isso, ela é traduzida por pesquisadores como “economia de bicos” e “economia sob demanda”. E está chegando a cada vez mais profissões no Brasil e no mundo, muito além de entregadores e motoristas.
+ 'Gig economy': o que é o trabalho que muda cada vez mais profissões no Brasil. Disponível em: https://www.otempo.com.br/economia/gig-economy-o-que-e-o-trabalho-que-muda-cada-vez-mais-profissoes-no-brasil-1.2881086. Acesso em: 25 out 2024.
+Uma das principais características da gig economy é a contratação de trabalhadores</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>independentes para tarefas específicas.</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>permanentes para tarefas específicas.</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>independentes para tarefas contínuas.</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>permanentes para tarefas contínuas.</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>temporários para tarefas contínuas.</t>
+        </is>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>A gig economy é caracterizada pela contratação de trabalhadores independentes para tarefas específicas, em vez de empregos permanentes e estáveis.</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K581" t="inlineStr"/>
+      <c r="L581" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Vários bairros de São Paulo enfrentam apagão após forte chuva
+Toda a cidade está em estado de atenção para alagamentos
+Vários bairros de São Paulo enfrentam um apagão por causa da forte chuva que atingiu a capital paulista no início da noite de hoje.
+Toda a cidade está em estado de atenção para alagamentos. Segundo o Centro de Gerenciamento de Emergências da capital paulista, pelos menos dois bairros estão com alerta para iminência de transbordamento.
+CBN. Disponível em: https://cbn.globo.com/sao-paulo/noticia/2024/10/11/varios-bairros-de-sao-paulo-enfrentam-apagao-apos-forte-chuva.ghtml. Acesso em: 16 out. 2024.
+Assinale a alternativa que identifica corretamente a preposição presente no trecho destacado e seu respectivo valor semântico:</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>"da", indicando posse.</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>"da", indicando tempo.</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>"por", indicando causa.</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>"por", indicando finalidade.</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>"da", indicando companhia.</t>
+        </is>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>A preposição "por" na expressão "por causa da" está corretamente indicando a causa do apagão, que é a forte chuva.</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K582" t="inlineStr"/>
+      <c r="L582" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Vários bairros de São Paulo enfrentam apagão após forte chuva
+Toda a cidade está em estado de atenção para alagamentos
+Vários bairros de São Paulo enfrentam um apagão por causa da forte chuva que atingiu a capital paulista no início da noite de hoje.
+Toda a cidade está em estado de atenção para alagamentos. Segundo o Centro de Gerenciamento de Emergências da capital paulista, pelos menos dois bairros estão com alerta para iminência de transbordamento.
+CBN. Disponível em: https://cbn.globo.com/sao-paulo/noticia/2024/10/11/varios-bairros-de-sao-paulo-enfrentam-apagao-apos-forte-chuva.ghtml. Acesso em: 16 out. 2024.
+O valor semântico do advérbio destacado indica</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>modo.</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>lugar.</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>tempo.</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>afirmação.</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>intensidade.</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>O advérbio hoje no trecho "início da noite de hoje" indica o tempo em que a forte chuva ocorreu, especificando que foi no mesmo dia em que o texto foi escrito.</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K583" t="inlineStr"/>
+      <c r="L583" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Montanhas no fundo do mar?
+A maior parte do mar profundo é plana e fica a, aproximadamente, 6 mil metros de profundidade, e essas regiões se estendem por milhões de quilômetros quadrados. Porém, nos locais onde ocorrem os encontros das placas tectônicas – grandes placas de rocha que se encaixam recobrindo toda a superfície da Terra – são formadas fendas enormes, que podem descer até 11 mil metros de profundidade.
+Disponível em: https://www.jornaljoca.com.br/colecao-tarsila-do-amaral-a-pintora-do-brasil-edicao-impressa-222/ Acesso em: 23 out. 2024.  
+A conjunção "porém" é substituída na oração sem perda semântica em:</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>"E, nos locais onde ocorrem os encontros das placas tectônicas"</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>"Porque, nos locais onde ocorrem os encontros das placas tectônicas"</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>"Embora, nos locais onde ocorrem os encontros das placas tectônicas"</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>"Portanto, nos locais onde ocorrem os encontros das placas tectônicas"</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>"Entretanto, nos locais onde ocorrem os encontros das placas tectônicas"</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>A conjunção "entretanto" é adversativa, assim como "porém". Ambas são usadas para introduzir uma ideia que contrasta com a anterior. No contexto da frase original, "porém" está sendo usado para mostrar um contraste em relação à informação sobre a maior parte do mar profundo ser plana. Substituir "porém" por "entretanto" mantém o mesmo valor semântico e a estrutura da frase, preservando o sentido original do texto.</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K584" t="inlineStr"/>
+      <c r="L584" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Leia este trecho de um artigo de opinião.
+Saúde mental nas escolas deve ser prioridade
+O tema da saúde mental no Brasil ganhou força no debate público nos últimos anos. Segundo o Observatório da Atenção Primária em Saúde, durante a pandemia de Covid-19 os casos de depressão aumentaram 41%. Quando o assunto é violência nas escolas, a Secretaria da Educação do Estado de São Paulo registrou 4.021 agressões físicas só nos dois primeiros meses do ano letivo de 2022— 48,5% a mais que no mesmo período de 2019, antes da crise sanitária.
+Mais do que delinear o cenário e diagnosticar os problemas, é preciso avançar em soluções propositivas para a saúde mental das(os) estudantes, seus responsáveis e educadoras(es), de forma estrutural. [..] A adolescência é uma fase propícia para ações de prevenção, cujos efeitos podem influenciar tanto o presente quanto o futuro.
+FREITAS, Rebeca; QUARTIERO, Maria Fernanda Resende; ALTENFELDER, Anna Helena. Saúde mental nas escolas deve ser prioridade. O Globo, 2 Jul 2022. Disponível em: https://oglobo.globo.com/opiniao/artigos/coluna/2022/07/saude-mental-nas-escolas-deve-ser-prioridade.ghtml. Acesso em: 16 out. 2024. (Adaptado). 
+No texto, os verbos em destaque estão no</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>pretérito perfeito e futuro do indicativo.</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>pretérito perfeito e presente do indicativo.</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>pretérito imperfeito e futuro do subjuntivo.</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>pretérito imperfeito e presente do indicativo.</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>pretérito mais que perfeito e futuro do indicativo.</t>
+        </is>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>Os verbos "ganhou", "aumentaram" e "registrou" estão no pretérito perfeito do indicativo, que indica uma ação concluída no passado. Já os verbos "é" e "podem" estão no presente do indicativo, que indica uma ação que ocorre no momento da fala.</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K585" t="inlineStr"/>
+      <c r="L585" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>As conjunções são palavras essenciais para a coesão e a fluidez de um texto. Elas podem ser classificadas em coordenativas e subordinativas. Exemplos de conjunções coordenativas incluem “e”, “mas” e “ou”, enquanto exemplos de conjunções subordinativas incluem “porque”, “quando” e “se”.
+Qual é a principal diferença entre conjunções coordenativas e subordinativas?</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Conjunções coordenativas são usadas apenas no início de frases, enquanto conjunções subordinativas são usadas no meio das frases.</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Conjunções coordenativas ligam orações independentes, enquanto conjunções subordinativas ligam orações dependentes.</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Conjunções coordenativas sempre indicam causa, enquanto conjunções subordinativas sempre indicam consequência.</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>Conjunções coordenativas indicam tempo, enquanto conjunções subordinativas indicam lugar.</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>Conjunções coordenativas são invariáveis, enquanto conjunções subordinativas são variáveis.</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>Conjunções coordenativas são usadas para ligar orações ou termos que têm a mesma função sintática e são independentes entre si. Por exemplo, em "Eu gosto de maçãs e ele gosta de laranjas", as orações são independentes. Por outro lado, conjunções subordinativas ligam uma oração principal a uma oração subordinada, que depende da principal para ter sentido completo. Por exemplo, em "Eu saí porque estava chovendo", a oração "porque estava chovendo" depende da principal para fazer sentido.</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K586" t="inlineStr"/>
+      <c r="L586" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>Leia o trecho abaixo para responder à questão.
+Minha terra tem palmeiras,
+Onde canta o Sabiá;
+As aves, que aqui gorjeiam,
+Não gorjeiam como lá.
+[...]
+DIAS, Gonçalves. Disponível em: http://www.dominiopublico.gov.br/download/texto/bn000100.pdf . Acesso em 06 jan. 2020.
+Do ponto de vista das classes gramaticais, as palavras em destaque no poema são classificadas como</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>pronomes espaciais.</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>locuções adjetivas.</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>advérbios de lugar.</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>locuções adverbiais.</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>advérbios de modo.</t>
+        </is>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>As palavras "onde", "aqui" e "lá" são advérbios de lugar. Advérbios são palavras que modificam o verbo, o adjetivo ou outro advérbio, indicando circunstâncias como tempo, modo, lugar, intensidade, entre outras. No caso específico do poema, "onde" indica o local em que algo acontece, "aqui" refere-se a um lugar próximo ao falante, e "lá" refere-se a um lugar distante do falante. Portanto, todas essas palavras estão relacionadas à indicação de lugares, caracterizando-se assim como advérbios de lugar.</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K587" t="inlineStr"/>
+      <c r="L587" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>Leia o trecho a seguir.
+Minha terra tem palmeiras,
+Onde canta o Sabiá;
+As aves, que aqui gorjeiam,
+Não gorjeiam como lá.
+[...]
+DIAS, Gonçalves. Disponível em: http://www.dominiopublico.gov.br/download/texto/bn000100.pdf . Acesso em 06 jan. 2020.
+Nos versos destacados, a expressão “como” é um(a)</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>advérbio que estabelece uma relação de lugar.</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>advérbio que estabelece uma relação de modo.</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>conjunção que estabelece uma relação causal.</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>conjunção que estabelece uma relação comparativa.</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>conjunção que estabelece uma relação de adição.</t>
+        </is>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>No poema, a palavra "como" desempenha o papel de conjunção estabelecendo uma relação comparativa. Nesse contexto, "como" está sendo utilizada para comparar o modo de gorjeio das aves em dois lugares diferentes: o lugar onde o eu lírico está (aqui) e o lugar ao qual ele se com saudade (lá).</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K588" t="inlineStr"/>
+      <c r="L588" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>Em relação à tirinha, assinale a alternativa que aponta para, respectivamente, um advérbio, um verbo e um adjetivo:</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>“outros”, “humanidade” e “tão”.</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>“lá”, “acham” e “difícil”.</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>“onde”, “pra” e “claro”.</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>“minha”, “que” e “é”.</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>“humanidade”, “estou” e “a”.</t>
+        </is>
+      </c>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>O termo "lá" é um advérbio de lugar, pois indica a localização de algo ou alguém em um ponto distante do falante. A palavra "acham" é um verbo, pois expressa uma ação realizada pelos sujeitos da frase. Já "difícil" é um adjetivo, pois qualifica um substantivo ao descrever a característica de algo que apresenta complexidade ou que não é fácil de ser realizado.</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K589" t="inlineStr">
+        <is>
+          <t>8a_ph02_por_08.png</t>
+        </is>
+      </c>
+      <c r="L589" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>Releia esta passagem do primeiro quadrinho:
+“Você só pode estacionar se me der 50 centavos.”.
+Os termos em destaque indicam que Calvin</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>fez uma proposta.</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>realizou uma persuasão.</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>impôs uma condição.</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>fez uma promoção.</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>fez uma exclusão.</t>
+        </is>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>No enunciado, os termos "só" e "se" indicam que Calvin está estabelecendo uma condição para que a ação de estacionar seja permitida. A palavra "só" limita a permissão, enquanto "se" introduz a condição necessária para que essa permissão seja concedida.</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K590" t="inlineStr">
+        <is>
+          <t>8a_ph02_por_09.png</t>
+        </is>
+      </c>
+      <c r="L590" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+A Educação Pela Pedra
+Uma educação pela pedra: por lições;
+para aprender da pedra, freqüentá-la;
+captar sua voz inenfática, impessoal
+(pela de dicção ela começa as aulas).
+A lição de moral, sua resistência fria
+ao que flui e a fluir, a ser maleada;
+a de poética, sua carnadura concreta;
+a de economia, seu adensar-se compacta:
+lições da pedra (de fora para dentro,
+cartilha muda), para quem soletrá-la.
+*
+Outra educação pela pedra: no Sertão
+(de dentro para fora, e pré-didática).
+No Sertão a pedra não sabe lecionar,
+e se lecionasse, não ensinaria nada;
+lá não se aprende a pedra: lá a pedra,
+uma pedra de nascença, entranha a alma.
+NETO, João Cabral de. A Educação Pela Pedra. Disponível em: http://www.academia.org.br/academicos/joao-cabral-de-melo-neto/textos-escolhidos. Acesso em: 15 jan. 2020.
+Observe os termos destacados no poema. Morfologicamente eles são classificados como</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>pronomes.</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>advérbios.</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>interjeições.</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>preposições.</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>adjetivos.</t>
+        </is>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>Morfologicamente os termos destacados são classificados como preposições, pois relacionam e conectam substantivos.</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K591" t="inlineStr"/>
+      <c r="L591" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>Manuela está jogando 2048, um jogo de quebra-cabeça onde o objetivo é combinar blocos com potências de 2 para formar blocos de maior valor. No tabuleiro, os blocos são sempre números que são potências de 2, como 2, 4, 8, 16 e assim por diante, conforme mostra a imagem.
+Disponível em: https://www.matematicagenial.com/2017/06/5-jogos-para-desenvolver-o-raciocinio-matematico.html.
+Para vencer, Manuela precisa combinar os blocos para formar o número 2048. Durante uma partida, ela fez uma série de movimentos e terminou com os blocos as potencias: 21 + 23+ 25 + 26 + 29. 
+Qual é a soma de todos os blocos do tabuleiro de Manuela em termos de potência de 2?</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>618</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>1024</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>A soma da potência 21 + 23+ 25 + 26 + 29 dos blocos é obtida por meio de:
+(2 × 1) + (2 × 2 × 2) + (2 × 2 × 2 × 2 × 2) + (2 × 2 × 2 × 2 × 2 × 2) + (2 × 2 × 2 × 2 × 2 × 2 × 2 × 2 × 2) = 618.</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K592" t="inlineStr">
+        <is>
+          <t>8a_ph02_mat_01.png</t>
+        </is>
+      </c>
+      <c r="L592" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>Um engenheiro está analisando a distância mínima entre a Terra e Júpiter para calcular a eficiência de painéis solares em uma estação espacial. A distância aproximada entre a Terra e Júpiter é de 591.000.000 km. Para simplificar os cálculos, ele precisa converter essa distância em notação científica.
+Qual é a forma correta dessa distância em notação científica?</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>59,1×108 km</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>59,1×105 km</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>59,1×106 km</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>5,91×108km</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>5,91×105 km</t>
+        </is>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>Para converter 591.000.000 em notação científica, desloca-se a vírgula 8 casas para a esquerda, mantendo como coeficiente apenas um algarismo, o que resulta em 5,91×108.</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K593" t="inlineStr"/>
+      <c r="L593" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>Um data center possui n racks de servidores, e cada rack contém n³ servidores. Sabendo que o total de servidores no data center é de 512, um engenheiro precisa determinar quantos racks de servidores o data center possui para planejar a expansão.
+Qual a quantidade de racks de servidores que possui o data center?</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>Se n é o número de racks, então n3  é o número de servidores por rack. O total de servidores é dado por n × n3. Portanto, n3 = 512. Calculando a ,3√ 512 temos que 
+Portanto, 512 = 23 · 23 · 23. Usando as propriedades da potenciação para escrever o radicando:</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K594" t="inlineStr"/>
+      <c r="L594" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>Em um estudo sobre o consumo de energia elétrica em uma cidade, os engenheiros precisam calcular a demanda total de energia de diferentes setores. A demanda de energia é representada pelas expressões 2,3 · 105 kWh para o setor residencial, 1,5 · 106 kWh para o setor comercial,  3,2 · 107 kWh para o setor industrial, e subtraída pela energia gerada por fontes renováveis, representada por  5 · 108 kWh. Eles precisam simplificar essa expressão para determinar a demanda total de energia.
+Qual é o resultado da expressão  ?</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>– 4,51 · 108</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>– 4,53 · 108</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>– 4,64 · 108</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>– 4,66  · 108</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>– 4,93 · 108</t>
+        </is>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>Somando e subtraindo as intensidades: 2,3 · 105 + 1,5 · 106  + 3,2 · 107  – 5 · 108 = (0,0023 + 0,015 + 0,32 – 5) · 108= – 4,66 · 108.</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K595" t="inlineStr">
+        <is>
+          <t>8a_ph02_mat_04.png</t>
+        </is>
+      </c>
+      <c r="L595" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>Em um estudo sobre crescimento populacional, os cientistas estão analisando a expressão para modelar a taxa de crescimento de uma população. Eles precisam simplificar essa expressão em forma de radical para entender melhor os dados.
+Qual é a forma simplificada da expressão ?</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>[img:8a_ph02_mat_05_a.png]</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>[img:8a_ph02_mat_05_b.png]</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>[img:8a_ph02_mat_05_c.png]</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>[img:8a_ph02_mat_05_d.png]</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>[img:8a_ph02_mat_05_e.png]</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>A expressão   pode ser simplificada como  , que é a forma correta em radical.</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K596" t="inlineStr">
+        <is>
+          <t>8a_ph02_mat_05.png</t>
+        </is>
+      </c>
+      <c r="L596" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>O tamanho de um átomo de hidrogênio é bem pequeno para os nossos parâmetros do dia a dia. Se aproximássemos o átomo ao formato de uma esfera, seu raio seria igual a 120 milionésimos de milionésimos de metro. A cada vez que falamos milionésimos, devemos dividir o número pela potência de 10 correspondente a milhão.
+Qual é o valor desse raio, em metros, escrito usando notação científica?</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>1,2 . 10-4</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>1,2 . 10-6</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>1,2 . 10-8</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>1,2 . 10-9</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>1,2 . 10-10</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>Primeiro, devemos calcular o que seria o milionésimo de milionésimo de metro: 1 metro deve ser dividido duas vezes por 106, potência correspondente a um milhão. Mas dividir por uma potência é o mesmo que multiplicar por uma potência de mesma base, mas o expoente deverá ter o sinal contrário. Logo:
+(1 ÷ 106) ÷ 106 = 1 ∙ 10-6 ∙ 10-6 = 1 ∙ 10-6+(-6) = 1 ∙ 10-12.
+A medida desejada é: 120 ∙ 10-12 m. Colocando 120 em notação científica, obtêm-se:
+120 ∙ 10-12 = (1,2 ∙ 102) ∙ 10-12 = 1,2 ∙102+(-12) = 1,2 ∙ 10-10 m.</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K597" t="inlineStr"/>
+      <c r="L597" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>Para determinar se uma raiz quadrada de um número natural é um número racional, devemos analisar o número que está dentro da raiz: o radicando. Observe os exemplos:
+, aqui o radicando é 4 e, como 4 é quadrado perfeito,  é racional.
+, aqui o radicando é 5 e, como 5 não é quadrado perfeito, não é racional.
+Dessa forma, considere os números  .</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Ambos são irracionais.</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>é irracional e  é racional</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>é racional e  é irracional.</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>Ambos são racionais.</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>Ambos são naturais.</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>é racional pois 36 é quadrado perfeito
+ é irracional pois 63 não é quadrado perfeito.</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K598" t="inlineStr">
+        <is>
+          <t>8a_ph02_mat_07.png</t>
+        </is>
+      </c>
+      <c r="L598" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>O PIB (produto interno bruto) do Brasil no 4º trimestre de 2016 foi de 1 630,6 Bilhões de reais. Como esse número ficará quando reescrito usando notação científica?</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>1,6306 . 103</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>1,6306 . 106</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>1,6306 . 109</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>1,6306 . 1012</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>1,6306 . 1015</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>A classe de bilhão corresponde a 109. Dessa forma, o número pode ser reescrito como:
+1 630,6 ∙ 109.
+Agora, colocando no formato de notação científica, será obtido: (1,6306 ∙ 103) ∙109.
+Usando as propriedades de potências: 1,6306 ∙10(3+9) = 1,6306 ∙ 1012.</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K599" t="inlineStr"/>
+      <c r="L599" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>Considere as 3 afirmações a seguir:
+I. 24 = (-2)4
+II. -35 = (-3)5;
+III. 43 = (-4)3.
+Quais das afirmações são verdadeiras?</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Apenas I.</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>I e II.</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>I e III.</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>II e III.</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>Apenas III.</t>
+        </is>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>I. 24 = 2 ∙ 2 ∙ 2 ∙ 2 = 16 e (-2)4 = (-2) ∙ (-2) ∙ (-2) ∙ (-2) = 16 (verdadeira);
+II. -35 = -3 ∙ 3 ∙ 3 ∙ 3 ∙ 3 = -243 e (-3)5 = (-3) ∙ (-3) ∙ (-3) ∙ (-3) ∙ (-3) = -243 (verdadeira);
+III. 43 = 4 ∙ 4 ∙ 4 = 64 e (-4)3 = (-4) ∙ (-4) ∙ (-4) = -64  (Falsa).</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K600" t="inlineStr"/>
+      <c r="L600" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>Leia um trecho sobre a notícia da primeira detecção de ondas gravitacionais:
+“... A colisão de buracos negros registrada pelo projeto foi detectada em 14 de setembro. Cada um dos dois objetos pesava cerca de 30 vezes a massa do Sol, e o fenômeno ocorreu a 1,3 bilhão de anos-luz.”
+Disponível em: http://g1.globo.com/ciencia-e-saude/noticia/2016/02/experimento-ve-ondas-gravitacionais-fenomeno-previsto-por-einstein.html. Acesso em: 10/01/2018.
+Ano-luz é uma medida de distância, usualmente utilizada em medidas astronômicas.
+Qual o valor dessa distância, em anos-luz, utilizando notação científica?</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>1,3 . 103</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>1,3 . 106</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>1,3 . 109</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>1,3 . 1012</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>1,3 . 1015</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>A classe de bilhão corresponde a 109. Dessa forma, o número pode ser reescrito como: 1,3 . 109.</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>PH02</t>
+        </is>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K601" t="inlineStr"/>
+      <c r="L601" t="inlineStr">
+        <is>
+          <t>8ano</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update questoes.xlsx: PH03, PH04
</commit_message>
<xml_diff>
--- a/questoes.xlsx
+++ b/questoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L601"/>
+  <dimension ref="A1:L651"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29844,7 +29844,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K552" t="inlineStr"/>
       <c r="L552" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -29969,7 +29968,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K554" t="inlineStr"/>
       <c r="L554" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -30028,7 +30026,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K555" t="inlineStr"/>
       <c r="L555" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -30087,7 +30084,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K556" t="inlineStr"/>
       <c r="L556" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -30145,7 +30141,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K557" t="inlineStr"/>
       <c r="L557" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -30204,7 +30199,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K558" t="inlineStr"/>
       <c r="L558" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -30262,7 +30256,6 @@
           <t>Ciências</t>
         </is>
       </c>
-      <c r="K559" t="inlineStr"/>
       <c r="L559" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -30448,7 +30441,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K562" t="inlineStr"/>
       <c r="L562" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -30507,7 +30499,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K563" t="inlineStr"/>
       <c r="L563" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -30566,7 +30557,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K564" t="inlineStr"/>
       <c r="L564" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -30625,7 +30615,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K565" t="inlineStr"/>
       <c r="L565" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -30684,7 +30673,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K566" t="inlineStr"/>
       <c r="L566" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -30810,7 +30798,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K568" t="inlineStr"/>
       <c r="L568" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -30939,7 +30926,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K570" t="inlineStr"/>
       <c r="L570" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31002,7 +30988,6 @@
           <t>Geografia</t>
         </is>
       </c>
-      <c r="K571" t="inlineStr"/>
       <c r="L571" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31063,7 +31048,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K572" t="inlineStr"/>
       <c r="L572" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31124,7 +31108,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K573" t="inlineStr"/>
       <c r="L573" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31185,7 +31168,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K574" t="inlineStr"/>
       <c r="L574" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31246,7 +31228,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K575" t="inlineStr"/>
       <c r="L575" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31307,7 +31288,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K576" t="inlineStr"/>
       <c r="L576" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31433,7 +31413,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K578" t="inlineStr"/>
       <c r="L578" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31494,7 +31473,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K579" t="inlineStr"/>
       <c r="L579" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31555,7 +31533,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K580" t="inlineStr"/>
       <c r="L580" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31616,7 +31593,6 @@
           <t>História</t>
         </is>
       </c>
-      <c r="K581" t="inlineStr"/>
       <c r="L581" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31679,7 +31655,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K582" t="inlineStr"/>
       <c r="L582" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31742,7 +31717,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K583" t="inlineStr"/>
       <c r="L583" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31803,7 +31777,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K584" t="inlineStr"/>
       <c r="L584" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31866,7 +31839,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K585" t="inlineStr"/>
       <c r="L585" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31925,7 +31897,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K586" t="inlineStr"/>
       <c r="L586" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -31990,7 +31961,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K587" t="inlineStr"/>
       <c r="L587" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -32055,7 +32025,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K588" t="inlineStr"/>
       <c r="L588" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -32259,7 +32228,6 @@
           <t>Português</t>
         </is>
       </c>
-      <c r="K591" t="inlineStr"/>
       <c r="L591" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -32384,7 +32352,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K593" t="inlineStr"/>
       <c r="L593" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -32444,7 +32411,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K594" t="inlineStr"/>
       <c r="L594" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -32632,7 +32598,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K597" t="inlineStr"/>
       <c r="L597" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -32759,7 +32724,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K599" t="inlineStr"/>
       <c r="L599" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -32823,7 +32787,6 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K600" t="inlineStr"/>
       <c r="L600" t="inlineStr">
         <is>
           <t>8ano</t>
@@ -32885,8 +32848,3106 @@
           <t>Matemática</t>
         </is>
       </c>
-      <c r="K601" t="inlineStr"/>
       <c r="L601" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>O clima da região Nordeste é semiárido, o que significa que o ano é dividido em estações chuvosas e estações de estiagem. A seca ocorre quando não chove nos meses em que deveria chover, no caso há expectativa de chuva entre janeiro e junho e ausência de precipitação esperada entre julho e dezembro.
+Disponível em: https://cienciahoje.periodicos.capes.gov.br/storage/acervo/ch/ch_308.pdf#page=43. Acesso em: 21 out. 2024. (Adaptado).
+Qual corrente oceânica tem influência direta no clima semiárido do sertão nordestino?</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Corrente do Golfo.</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Corrente das Falklands.</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Corrente do Brasil.</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>Corrente de Humboldt.</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>Corrente de Benguela.</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>A Corrente do Brasil é uma corrente quente que flui ao longo da costa leste do Brasil e influencia diretamente o clima da região Nordeste, contribuindo para a variabilidade das chuvas.</t>
+        </is>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K602" t="inlineStr"/>
+      <c r="L602" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>O encontro das correntes marinhas do Brasil e das Malvinas em região adjacente, o fenômeno da ressurgência (em que a água do fundo oceânico, fria e rica em plâncton, sobe à superfície) e a influência da pluma do rio da Prata permitem o aparecimento de peixes e crustáceos de ambientes tropicais e de pinguins e baleias-francas, de clima subtropical.
+Disponível em: https://cienciahoje.periodicos.capes.gov.br/storage/acervo/ch/ch_313.pdf#page=37. Acesso em: 21 out. 2024. (Adaptado).
+Qual é a principal consequência do fenômeno da ressurgência na costa brasileira?</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Diminui a temperatura da água, tornando-a imprópria para a maioria das espécies comerciais.</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Aumenta a concentração de nutrientes, favorecendo a proliferação de espécies marinhas.</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Reduz a salinidade da água, afetando negativamente a reprodução de peixes.</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>Provoca a migração de espécies tropicais para águas mais profundas.</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>Causa a formação de zonas mortas, onde a vida marinha é escassa.</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>A ressurgência traz água rica em nutrientes para a superfície, o que favorece a proliferação de plâncton e, consequentemente, de outras espécies marinhas.</t>
+        </is>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K603" t="inlineStr"/>
+      <c r="L603" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>Mudanças climáticas afetam diretamente a biodiversidade de uma região, já que algumas espécies são bastante sensíveis à variação de temperatura. Os corais recifais, por exemplo, não se adaptam a águas muito geladas.
+Disponível em: https://cienciahoje.periodicos.capes.gov.br/storage/acervo/ch/ch_283.pdf#page=63. Acesso em: 21 out. 2024. (Adaptado).
+Como a Corrente do Brasil pode impactar os recifes de corais na costa brasileira?</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Diminuindo a temperatura da água e protegendo os corais do branqueamento.</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Aumentando a temperatura da água e elevando o branqueamento dos corais.</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>Diminuindo a acidez da água e exacerbando o branqueamento dos corais.</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>Reduzindo a salinidade da água e favorecendo a recuperação dos corais.</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>Aumentando a acidez da água e protegendo os corais.</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>A Corrente do Brasil é uma corrente quente que pode aumentar a temperatura da água, contribuindo para o branqueamento dos corais.</t>
+        </is>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K604" t="inlineStr"/>
+      <c r="L604" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>Um sapo está dentro de uma panela sobre o fogo. A água aquece lentamente e o animal não percebe o aumento da temperatura até não se mais capaz de sair da panela e se livrar da morte. A história foi usada no 1º Encontro do Painel Intergovernamental de Mudanças do Clima (IPCC) na América Latina para ilustrar o comportamento da humanidade em relação às mudanças climáticas.
+Disponível em: https://cienciahoje.periodicos.capes.gov.br/storage/acervo/ch/ch_244.pdf#page=48. Acesso em: 21 out. 2024. (Adaptado).
+Segundo a analogia proposta no texto, qual é a consequência das mudanças climáticas para a biodiversidade?</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Aumento da diversidade de espécies de águas frias.</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Proliferação de espécies exóticas.</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Destruição de habitats e redução da biodiversidade.</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>Expansão de espécies de águas profundas.</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>Aumento da resistência das espécies às mudanças ambientais.</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>As mudanças climáticas levam à destruição de habitats naturais, resultando em uma redução da biodiversidade.</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K605" t="inlineStr"/>
+      <c r="L605" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>Nas últimas décadas, a poluição da atmosfera aumentou bastante por conta da queima de combustíveis das indústrias e dos automóveis. A derrubada de árvores para fabricação de papel, móveis e outros materiais também é muito prejudicial ao meio ambiente. Fatores como esses contribuem para um processo de mudanças climáticas globais, ou seja, um conjunto de alterações em determinadas características do clima do planeta.
+Disponível em: https://cienciahoje.periodicos.capes.gov.br/storage/acervo/chc/chc_214.pdf#page=06. Acesso em: 21 out. 2024.
+Qual dos seguintes eventos climáticos extremos recentes no Brasil pode ser diretamente associado a essas mudanças climáticas?</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Aumento da biodiversidade na Amazônia.</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Redução das áreas de desertificação no Nordeste.</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Intensificação das chuvas e enchentes no Sudeste.</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>Diminuição das temperaturas médias no Sul.</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>Estabilização dos níveis dos rios no Centro-Oeste.</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>As mudanças climáticas podem levar a eventos climáticos extremos, como chuvas intensas e enchentes.</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K606" t="inlineStr"/>
+      <c r="L606" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>João comentou com seu amigo, José, que o clima desse fim de semana seria de muito sol e calor.
+Em relação aos conceitos de clima e tempo, a análise de João para o fim de semana está:</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>correto, pois clima se relaciona com as condições atmosféricas momentâneas.</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>correto, pois clima se relaciona com as condições atmosféricas ao longo de anos.</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>incorreto, pois clima se relaciona com as condições atmosféricas ao longo de anos.</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>incorreto, pois clima se relaciona com as condições atmosféricas momentâneas.</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>correto, pois clima e tempo são sinônimos e não há diferenças.</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>João está se referindo ao tempo, o qual se refere às condições atmosféricas momentâneas. O termo clima faz referência às condições atmosféricas de um local ao longo de anos.</t>
+        </is>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K607" t="inlineStr"/>
+      <c r="L607" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>Uma mudança climática, por exemplo, afeta diretamente a biodiversidade de uma região, já que algumas espécies são bastante sensíveis à variação de temperatura. Os corais recifais, por exemplo, não se adaptam a águas muito geladas.
+Disponível em: https://cienciahoje.periodicos.capes.gov.br/storage/acervo/ch/ch_283.pdf#page=63. Acesso em: 06 dez 2024.
+Com base no texto que afirma que "algumas espécies são bastante sensíveis à variação de temperatura", analise as alternativas abaixo e escolha aquela que melhor exemplifica um impacto direto do aumento da temperatura na biodiversidade.</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>aumento da temperatura pode favorecer a proliferação de espécies invasoras.</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>redução da temperatura pode aumentar a produtividade agrícola.</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>aumento da temperatura pode reduzir a incidência de doenças em plantas.</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>redução da temperatura pode aumentar a diversidade de espécies aquáticas.</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>aumento da temperatura pode diminuir a taxa de evaporação dos corpos d'água.</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>O aumento da temperatura pode favorecer a proliferação de espécies invasoras. Com a intensificação do aquecimento global, muitas espécies invasoras encontram condições ideais para se proliferar, o que pode desestabilizar ecossistemas locais e afetar a biodiversidade.</t>
+        </is>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K608" t="inlineStr"/>
+      <c r="L608" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>Ferramenta prevê influência do clima sobre agricultura em 2018
+Lançado em agosto de 2016 pela Escola Superior de Agricultura Luiz de Queiroz (Esalq) da USP em Piracicaba, o Sistema TempoCampo finalizou o ano de 2017 com projeções climáticas para 2018.
+Criado no Departamento de Engenharia de Biossistemas da Esalq, o Sistema TempoCampo é resultado da intersecção de diversos projetos de pesquisa na área de modelagem agrícola e agrometeorologia. Com um banco de dados climáticos para todos os Estados brasileiros, o sistema oferece aos produtores a possibilidade de antever os efeitos do clima sobre determinadas culturas ao longo das safras. É possível saber, assim, se elas serão favorecidas ou prejudicadas por fatores meteorológicos.(...)
+Disponível em: &lt;https://jornal.usp.br/universidade/ferramenta-preve-influencia-do-clima-sobre-agricultura-em-2018/&gt;. Acesso em: 2 set. 2018.
+O texto aborda um assunto de grande importância para os produtores agrícolas que é</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>a melhor semente a ser plantada para conseguir germinar em qualquer tipo de clima.</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>a melhor época do ano para se plantar determinadas espécies de legumes e verduras.</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>o estudo da meteorologia para prever as possíveis mudanças climáticas para auxiliar em possíveis mudanças prejudiciais para a agricultura.</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>a quantidade de água que a plantação terá acesso naquele ano para decidir o melhor tipo de alimento a ser plantado naquele ano.</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>o estudo da meteorologia para prever as possíveis mudanças no tempo para alertar os trabalhadores rurais.</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>A reportagem traz uma novidade tecnológica que é uma ferramenta que pode prever mudanças climáticas. Isso auxilia os agricultores a preparar suas lavouras e minimizar os impactos e perdas.</t>
+        </is>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K609" t="inlineStr"/>
+      <c r="L609" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>Os recifes de corais são ecossistemas extremamente importantes para a biodiversidade marinha, sendo fonte de alimento e abrigo para uma variedade de espécies. No Brasil, esses recifes estão principalmente no litoral nordestino, e o Parque Nacional Marinho dos Abrolhos é um exemplo de área protegida dedicada à conservação desse ecossistema. No entanto, os recifes brasileiros têm enfrentado grandes desafios, como o branqueamento dos corais, causado pelo aumento das temperaturas dos oceanos devido às mudanças climáticas.
+Considerando a função dos recifes de corais nos ecossistemas marinhos, qual é o impacto ecológico mais provável do branqueamento de corais na biodiversidade?</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>O branqueamento dos corais estimula a colonização de novas espécies, aumentando a diversidade.</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>A perda das algas simbióticas enfraquece os corais, reduzindo o alimento e abrigo para várias espécies.</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>O branqueamento diminui a diversidade temporariamente, mas aumenta o crescimento de algas.</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>O branqueamento protege os corais contra predadores, ajudando na recuperação dos recifes.</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>A perda de pigmentação do coral não interfere na biodiversidade, pois afeta apenas a cor do recife.</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>Sem as algas simbióticas, os corais enfraquecem, perdendo a capacidade de suportar uma alta biodiversidade.</t>
+        </is>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J610" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K610" t="inlineStr"/>
+      <c r="L610" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>O Pantanal, a maior planície alagável do mundo, é um dos biomas com a maior biodiversidade do planeta. Ele passa por um ciclo anual de cheias e secas, o que cria um ambiente fértil e variado que sustenta muitas espécies. No entanto, as atividades humanas, como a agricultura, a pecuária e o desmatamento, estão causando degradação ambiental no Pantanal, ameaçando o equilíbrio ecológico e a diversidade de espécies.
+Qual das alternativas abaixo descreve melhor como o ciclo natural de cheias e secas do Pantanal beneficia a biodiversidade local?</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>O ciclo de cheias e secas aumenta a salinidade do solo, favorecendo espécies adaptadas ao sal.</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>As cheias anuais distribuem nutrientes no solo, criando habitats variados que sustentam muitas espécies.</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>O período de seca elimina as espécies menos adaptadas, fortalecendo a biodiversidade.</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>As secas constantes reduzem a vegetação, permitindo a sobrevivência de espécies aquáticas.</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>O ciclo de cheias e secas é responsável por criar um solo infértil, limitando o crescimento da vegetação.</t>
+        </is>
+      </c>
+      <c r="G611" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>O ciclo natural de cheias e secas do Pantanal é fundamental para a manutenção da sua biodiversidade. Durante as cheias, os rios transbordam e inundam grandes áreas, depositando sedimentos ricos em nutrientes no solo. Esses nutrientes são essenciais para o crescimento de diversas plantas, que por sua vez sustentam uma ampla variedade de animais. Além disso, as cheias criam diferentes tipos de habitats, como áreas alagadas, lagoas temporárias e campos secos, que abrigam diferentes espécies de flora e fauna. Esse mosaico de habitats permite que muitas espécies coexistam, aumentando a biodiversidade do bioma.</t>
+        </is>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J611" t="inlineStr">
+        <is>
+          <t>Ciências</t>
+        </is>
+      </c>
+      <c r="K611" t="inlineStr"/>
+      <c r="L611" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>Disponível em: https://images.populationpyramid.net/capture/?selector=%23pyramid-share-container&amp;url=https%3A%2F%2Fwww.populationpyramid.net%2Fpt%2Fcanad%25C3%25A1%2F2023%2F%3Fshare%3Dtrue. Acesso em: 24 set. 2024.
+A partir da pirâmide etária do Canadá em 2023, é possível destacar que este país possui como característica</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>uma possível redução de trabalhadores no futuro.</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>a existência de  muitos jovens e alta taxa de fecundidade.</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>uma menor parcela da população entre homens e mulheres.</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>a baixa expectativa de vida da população para o futuro.</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>uma predominância da população idosa.</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>A pirâmide etária do Canadá em 2023 mostra que a faixa etária "0-4 anos" possui a menor proporção da população. Isso indica que pode haver uma redução na quantidade de jovens entrando no mercado de trabalho no futuro, potencialmente resultando em uma escassez de trabalhadores.</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K612" t="inlineStr">
+        <is>
+          <t>8a_ph03_geo_01.jpg</t>
+        </is>
+      </c>
+      <c r="L612" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+A Estátua da Liberdade, um dos grandes símbolos dos EUA, desde 1886 "guarda" a entrada de Nova York pelo mar. [...]  A obra voltou ao imaginário americano depois da publicação dos controversos planos do presidente Donald Trump para a imigração, em especial sua tentativa de vetar a entrada de indivíduos de sete países majoritariamente muçulmanos - que atribui a questões de segurança.
+Disponível em: https://www.bbc.com/portuguese/internacional-38919713#:~:text=Objeto%20de%20controv%C3%A9rsia&amp;text=%22E%20se%20uma%20imagem%20ocidental,o%20projeto%20ser%20rejeitado%20totalmente.%22&amp;text=Esta%20n%C3%A3o%20foi%20a%20%C3%BAnica,correntes%20quebradas%2C%20al%C3%A9m%20da%20tocha. Acesso em 24 de out de 2024.
+Qual é o simbolismo principal da Estátua da Liberdade, inaugurada em 1886 em Nova York, especialmente ressaltado pelo poema gravado em sua base?</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Comemorar a vitória americana na Guerra Civil.</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Marcar a aliança entre os Estados Unidos e a França.</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Exprimir solidariedade e acolhimento a imigrantes e estrangeiros.</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>Representar a inovação em monumentos de obras arquitetônicas pelo globo.</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>Representar a maioridade política dos Estados Unidos no cenário internacional.</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>Inaugurada em 1886, a Estátua da Liberdade guarda a entrada de Nova York pelo mar e simboliza a promessa feita aos imigrantes na época: liberdades civis, iniciativa privada e oportunidades de trabalho. O poema na base da estátua exalta a solidariedade e o acolhimento aos imigrantes, um tema que voltou ao imaginário americano durante os controversos planos do presidente Donald Trump para a imigração.</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K613" t="inlineStr"/>
+      <c r="L613" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+Ao longo do último meio século, o Canadá se transformou em uma nação multicultural. Com uma imensa área habitada por apenas 12 milhões de pessoas após a 2ª Guerra Mundial, o governo canadense promoveu políticas durante as décadas seguintes para atrair estrangeiros.
+Além de tornar o Canadá uma das sociedades mais multiculturais do mundo, a imigração tem sido um motor do crescimento.
+Disponível em: https://www.bbc.com/portuguese/articles/c4nx08pp0q1o. Acesso em: 24 out. 2024. 
+Qual é o principal motivo pelo qual o Canadá promove políticas de imigração?</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Atrair trabalhadores para o mercado de trabalho e expandir a economia.</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Promover a sua imagem internacional como um país acolhedor.</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Fortalecer o sistema educacional com a diversidade cultural.</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>Criar alianças estratégicas com outros países.</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>Incrementar o setor turístico e cultural no país.</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>Ao longo do último meio século, o Canadá se tornou uma nação multicultural. Após a 2ª Guerra Mundial, com uma população de apenas 12 milhões de pessoas, o governo canadense implementou políticas para atrair estrangeiros com o objetivo de povoar o país e expandir sua economia. A imigração tem sido um motor do crescimento, trazendo talento e mão de obra para as empresas canadenses.</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K614" t="inlineStr"/>
+      <c r="L614" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>Disponível em: http://www.geografia.seed.pr.gov.br/modules/galeria/detalhe.php?foto=1529&amp;evento=5. Acesso em 25 de out de 2024.
+Quais países compõem a América Anglo-Saxônica?</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Estados Unidos e Canadá.</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>México e Estados Unidos.</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>México e Guatemala.</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>Canadá e México.</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>Brasil e Argentina.</t>
+        </is>
+      </c>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>No mapa, a América Anglo-Saxônica está representada pela região em vermelho, que é composta pelos Estados Unidos e Canadá. Essa área é caracterizada pelo predomínio da língua inglesa e da cultura de origem britânica.</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K615" t="inlineStr">
+        <is>
+          <t>8a_ph03_geo_04.jpg</t>
+        </is>
+      </c>
+      <c r="L615" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+Os colonizadores estabeleceram o conceito de raça com base em fenótipos e cor da pele para classificar os seres humanos. Eles se autodenominaram brancos e consideraram aqueles que não eram brancos como pertencentes a raças inferiores, passíveis, portanto, de serem subjugados, escravizados e/ou explorados. Os Estados Unidos da América foram construídos sobre a divisão racial, com quase 250 anos de nação sustentados pela hierarquia racial.
+Disponível em: https://www.opeu.org.br/2024/06/08/racismo-institucional-nos-eua-o-caso-raven-baxter-e-a-persistencia-da-discriminacao-racial/. Acesso em 24 de out de 2024.
+Qual foi o papel da hierarquia racial na formação dos Estados Unidos?</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Permitiu a emancipação de diferentes grupos étnicos no país.</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Teve influência insignificante na formação dos Estados Unidos.</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Destinou-se para manter a segregação e a desigualdade entre as raças.</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Contribuiu para fortalecer os pilares de igualdade e liberdade no país.</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>Caminhou para fortalecer os distintos laços entre diferentes culturas.</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>A hierarquia racial nos Estados Unidos moldou profundamente a estrutura social, econômica e política do país. Embora tenham sido feitos progressos significativos na luta contra a discriminação racial, os efeitos dessa hierarquia ainda são visíveis e continuam a influenciar a sociedade americana.</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K616" t="inlineStr"/>
+      <c r="L616" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>Leia o texto a seguir.
+Megalópole
+José Horta Nunes
+A nomeação megalópole significa a cidade pela sua grandeza e influência, e nessa direção, ela funciona como sinônimo de metrópole. A megalópole significa também um grande aglomerado de cidades, resultante do crescimento e da junção delas, ou seja, de uma conurbação. Com a fusão das cidades, o espaço rural fica bastante delimitado, ao pondo em alguns casos de a distinção urbano x rural não funcionar mais.
+Um caso típico, apontado por vários urbanistas, é o da megalópole de Boswash, que vai de Boston a Washinton, no Nordeste dos Estados Unidos. Inclui as metrópoles de Nova York, Filadélfia, Baltimore e Washington. No Brasil, está em formação uma megalópole que une as regiões metropolitanas do Rio de Janeiro e de São Paulo, estendo-se até a região metropolitana de Campinas.
+[...]
+Disponível em:&lt; https://www.labeurb.unicamp.br/endici/index.php?r=verbete%2Fview&amp;id=237&gt;. Acesso em: 18 mar. 2020.
+A região em que se localiza BosWash é conhecida como:</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Grandes lagos.</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Nordeste.</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Costa sul.</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Planícies centrais.</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>Montes apalaches.</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>Sendo uma das maiores megalópoles do mundo, BosWash está localizada nas áreas urbanas de maior desenvolvimento no Nordeste dos Estados Unidos.</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K617" t="inlineStr"/>
+      <c r="L617" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>Um homem atropelou várias pessoas neste sábado (12) em uma marcha de manifestantes antirracismo em Charlottesville, na Virgínia. A cidade está sendo palco de conflitos entre esses ativistas e manifestantes nacionalistas brancos, neonazistas e membros da Ku Klux Klans que se reuniram desde a noite de sexta-feira (11)[...] Segundo as autoridades, uma mulher de 32 anos morreu no atropelamento. Outras 19 pessoas ficaram feridas --cinco estão em estado crítico. Além dessa morte, um helicóptero da polícia caiu, deixando dois mortos --a polícia investiga as causas e se o caso tem relação direta com o conflito racial.
+[...]
+UOL SP. Suspeito é preso após atropelar multidão e matar manifestante em marcha antirracismo nos EUA. 12 ago.2017. Disponível
+em:https://noticias.uol.com.br/internacional/ultimas-noticias/2017/08/12/carro-atropela-manifestantes-durante-protesto-desupremacistas-brancos-nos-eua.htm. Acesso em: 16 mar.2020
+Atentados racistas podem ser explicados pela</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>diminuição do nacionalismo branco.</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>tentativas de se reimplantar a escravidão.</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>radicalismo cristão que prega a hierarquia social.</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>autossegregação dos negros em relação aos brancos.</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>permanência de políticas segregacionistas pós-escravidão.</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>Mesmo após o fim da escravidão, permaneceram práticas segregacionistas semelhantes ao apartheid da África do Sul, desta forma, o conflito e o ideal de superioridade étnica perduram até hoje nos EUA, tendo se intensificado nos últimos anos.</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K618" t="inlineStr"/>
+      <c r="L618" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>A porta-voz da Casa Branca, Sarah Sanders, defendeu nesta o presidente Donald Trump das acusações de que ele estimulou a violência contra uma deputada muçulmana, depois de tuitar um vídeo que alterna imagens da parlamentar e dos ataques de 11 de setembro de 2001.
+A declaração de Sanders veio logo depois de a presidente da Câmara dos Deputados, a democrata Nancy Pelosi, dizer que conversou com as autoridades sobre a segurança de sua colega e pedir a Trump que apagasse o tuíte.
+No post, o presidente americano compartilhou um vídeo em que a congressista Ilhan Omar fala sobre o 11 de setembro. A edição foi feita de forma que a declaração da deputada é repetida e alternada com cenas dos atentados.
+[...]
+REDAÇÃO. Revista Veja. Trump é acusado de estimular violência contra deputada muçulmana. 15 abr.2019. Disponível
+em:&lt;https://veja.abril.com.br/mundo/trump-e-acusado-de-estimular-violencia-contra-congressista-muculmana/.&gt; Acesso em: 17mar. 2020.
+Imigrantes residentes nos EUA de origem islâmica sofrem com um estereótipo relacionado</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>a prática de crimes.</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>a intolerância cultural.</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>a atentados terroristas.</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>ao baixo nível de instrução.</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>a falta de protagonismo feminino.</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>Em 2001 atentados terroristas provocados por grupos islâmicos mataram cerca de 3 mil pessoas nos EUA, desde então, pessoas e grupos de origem islâmica sofrem com o estereótipo de terroristas.</t>
+        </is>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K619" t="inlineStr"/>
+      <c r="L619" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>Considerando que os EUA estão na terceira fase de transição demográfica, é característica deste país nos tempos atuais:</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>As altas taxas de mortalidade infantil.</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>A farta disponibilidade de mão-de-obra.</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>O significativo incremento da imigração.</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>As altas taxas de crescimento demográfico.</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>O progressivo envelhecimento populacional.</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>A terceira fase da transição demográfica caracteriza-se por baixos valores de crescimento demográfico, onde a baixa natalidade e a melhoria das condições de saúde geram envelhecimento populacional.</t>
+        </is>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J620" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K620" t="inlineStr"/>
+      <c r="L620" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>Os jovens que uniram indígenas dos EUA contra oleoduto barrado por Obama e liberado por Trump
+A celebração pôs fim a uma das maiores mobilizações de indígenas americanos em várias décadas[...]
+[...]
+Mas quando começou, em abril, o movimento não passava de um "acampamento de reza" erguido por um punhado de jovens e adolescentes sioux à beira do rio Cannonball.
+[...]
+Defensores do projeto dizem que ele gerará empregos na indústria petrolífera, reduzirá a dependência dos EUA por importações de combustíveis e barateará a gasolina.
+[...]
+FELLETE, João. Os jovens que uniram indígenas dos EUA contra oleoduto barrado por Obama e liberado por Trump. Da BBC Brasil em
+Washington. Disponível em:&lt; https://www.bbc.com/portuguese/internacional-38926624&gt;. Acesso em: 18 mar.2020.
+O contexto dado assemelha-se ao ideal pós-colonial de ocupação do território estadunidense na medida em que</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>concebe ao território prioridade econômica.</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>sempre respeitam as decisões nacionais indígenas.</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>prioriza a intocabilidade ambiental.</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>busca efetivar a consolidação do estado-nacional.</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>oferta terras a imigrantes britânicos.</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>Ainda hoje a prioridade dada ao território é de cunho econômico, o que gera conflito com visões não predatórias típicas das comunidades indígenas. Fenômeno que se processa desde tempos coloniais.</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>Geografia</t>
+        </is>
+      </c>
+      <c r="K621" t="inlineStr"/>
+      <c r="L621" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>A própria noção de Iluminismo, Ilustração, ou ainda Esclarecimento, como o termo é por vezes traduzido, indica, através da metáfora da luz e da claridade, uma oposição às trevas, ao obscurantismo, á ignorância, à superstição, ou seja, à existência de algo oculto, enfatizando, ao contrário, a necessidade de o real, em todos os seus aspectos, tornar-se transparente à razão. 
+MARCONDES, Danilo. Iniciação a História da Filosofia: Dos Pré-Socráticos a Wittgenstein. Rio de Janeiro: Jorge Zahar, 2018, p. 207.
+A metáfora da luz trazida pelo Iluminismo se dá em oposição às "trevas" da(do)</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Idade Média, compreendida de forma negativa pelos Iluministas que rejeitavam o dogmatismo religioso característico desse período.</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Democracia, percebida como uma estrutura de poder injusta e arbitrária pelos pensadores iluministas.</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Revolução Científica, rejeitada pelos iluministas por ter incentivado o abandono das práticas do cristianismo.</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Renascimento, visto como herege por ter deslocado o centro das artes da esfera religiosa para os aspectos humanos</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>Antigo Regime, entendido como a estrutura responsável por desestruturar o feudalismo defendido pelos iluministas.</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>Os iluministas frequentemente viam a Idade Média como uma época de trevas, dominada pela ignorância e pela superstição, em oposição às ideias de razão e esclarecimento do Iluminismo.</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J622" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K622" t="inlineStr"/>
+      <c r="L622" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>Conhecido como o século das Luzes ou do Iluminismo, o século XVIII foi marcado por um movimento do pensamento europeu (ocorrido mais especificamente na segunda metade do século XVIII) que abrangeu o pensamento filosófico e gerou uma grande revolução nas artes (principalmente na literatura), nas ciências, nos costumes, na teoria política e na doutrina jurídica. O Iluminismo também se distinguiu pela centralidade da ciência e da racionalidade crítica no questionamento filosófico.
+Disponível em: https://www.maxwell.vrac.puc-rio.br/15543/15543_3.PDF. Acesso em: 22 out. 2024
+O movimento mencionado no texto teve como principal característica a</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>rejeição completa da religião e a adoção do ateísmo como doutrina oficial das sociedades europeias.</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>promoção de revoluções exclusivamente políticas sem impacto em outras áreas do conhecimento.</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>centralidade da ciência e da racionalidade crítica no questionamento filosófico.</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>priorização do ensino religioso como forma de produção de conhecimento.</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>ênfase na manutenção das tradições e dogmas medievais.</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>O Iluminismo enfatizou o uso da razão e da ciência para questionar e reformar todas as áreas do conhecimento humano, incluindo a filosofia, as artes, as ciências, os costumes, a teoria política e a doutrina jurídica. Este movimento foi fundamental para o desenvolvimento do pensamento crítico e científico.</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J623" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K623" t="inlineStr"/>
+      <c r="L623" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>Galileu Galilei nasceu na cidade de Pisa em 1564, mesmo ano da morte do pintor e escultor Michelangelo e do nascimento do dramaturgo inglês William Shakespeare. Exatos 31 anos antes, o matemático e astrônomo polonês Nicolau Copérnico publicou sua obra maior – Das revoluções dos corpos celestes –, defendendo a teoria de que a Terra se move em torno do Sol, e não o contrário.
+Essa teoria seria defendida e desenvolvida por Galileu e seu contemporâneo Johannes Kepler, que primeiro descreveu a trajetória elíptica dos planetas. A síntese final desses trabalhos foi a Teoria da Gravitação Universal, formulada pelo físico e matemático inglês Isaac Newton que, por coincidência, nasceu em 1642, o mesmo ano em que Galileu morreu.
+CAVALCANTE, Pedro. Como Galileu inventou a ciência moderna. Disponível em: https://super.abril.com.br/historia/o-novo-mundo-de-galileu. Acesso em: 22 out. 2024.
+A teoria concebida por Copérnico e desenvolvida por Galileu e Kepler deu origem ao</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>humanismo.</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>heliocentrismo.</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>protestantismo.</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>iluminismo.</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>geocentrismo.</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>A teoria defendida por Copérnico, e depois desenvolvida por Galileu e Kepler, é conhecida como heliocentrismo. Ela propõe que a Terra e os outros planetas giram em torno do Sol, desafiando a visão geocêntrica tradicional que colocava a Terra no centro do universo.</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K624" t="inlineStr"/>
+      <c r="L624" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>A efervescência cultural da Renascença criara uma vaga que não cessava de afogar as velhas certezas da Filosofia e da ciência baseadas sobretudo nos escritos do grego Aristóteles e na autoridade da Bíblia. O prestígio do Estado e da Igreja estavam igualmente corroídos pela dissidência política e pela Reforma protestante. Um novo mundo nascia. Mesmo em retirada, porém, a velhas instituições permaneciam, no início do século XVII, robustas o suficiente para queimar na fogueira um certo número de pensadores atrevidos.
+Descartes: a razão acima de tudo. Disponível em: https://super.abril.com.br/comportamento/descartes-a-razao-acima-de-tudo?utm_source=google&amp;utm_medium=cpc&amp;utm_campaign=eda_super_audiencia_institucional-Performance-Max-nova&amp;gad_source=1&amp;gclid=Cj0KCQjwmt24BhDPARIsAJFYKk0YMLGXm1apAQs1wxRQ_szSQzKsgCJJ8I_RXCnww8Lb4_A6gF-HnO4aAgx2EALw_wcB. Acesso em: 22 out. 2024.
+Como a Revolução Científica desafiou as antigas instituições, e qual foi a consequência enfrentada pelos cientistas?</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>A Revolução Científica reafirmou as teorias de Aristóteles, resultando no apoio incondicional da igreja aos novos cientistas.</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Os cientistas passaram a questionar explicações baseadas na religião, resultando em perseguições e punições severas promovidas pela igreja.</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>A Revolução Científica eliminou todas as tradições religiosas, levando a uma cooperação harmoniosa entre a igreja e os cientistas.</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Os seus pensadores fixaram suas formulações na Bíblia e na tradição, levando ao desenvolvimento conjunto de cientistas e teólogos.</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>O Estado incentivou os cientistas a colaborarem com a igreja para desenvolver novas tecnologias, resultando na aceitação plena das descobertas científicas.</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>Durante a Revolução Científica, os estudiosos começaram a desafiar as explicações tradicionais apoiadas pela igreja, o que levou a muitos conflitos, perseguições e até execuções de cientistas, como uma forma de suprimir tais ideias que desafiavam a autoridade religiosa.</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K625" t="inlineStr"/>
+      <c r="L625" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>Seu maior legado, porém, não foi uma descoberta científica específica, e sim um jeito de pensar. Galileu insistiu que a linguagem adequada para a filosofia natural (o nome que se dava, na época, às ciências exatas e biológicas) era a matemática, e não a palavra. Que qualquer afirmação sobre a natureza deveria partir da observação da própria natureza. Que é preciso acumular dados e fazer experimentos. 
+CAVALCANTE, Pedro. Como Galileu inventou a ciência moderna. Disponível em: https://super.abril.com.br/historia/o-novo-mundo-de-galileu. Acesso em: 23 out. 2024.
+Qual foi o principal legado de Galileu Galilei para a filosofia natural, conforme descrito no texto?</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Desenvolvimento de hipóteses filosóficas com base exclusivamente na tradição e nos textos sagrados.</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Aplicação rigorosa do método científico, enfatizando a observação, a experimentação e o uso da matemática.</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Rejeição do uso da matemática na filosofia natural, priorizando a linguagem poética e literária.</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Defesa da supremacia das explicações teológicas sobre as científicas, seguindo os dogmas da igreja.</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>Promoção do pensamento especulativo sem a necessidade de experimentação ou acumulação de dados.</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>O principal legado de Galileu foi a defesa da abordagem científica baseada na observação direta da natureza, no acúmulo de dados e na experimentação, utilizando a matemática como linguagem para descrever os fenômenos naturais, elementos centrais do método científico.</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J626" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K626" t="inlineStr"/>
+      <c r="L626" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>O pensamento iluminista, baseado no racionalismo, individualismo e liberdade absoluta do homem, ao criticar todos os fundamentos em que se assentava o Antigo Regime, revelava as suas contradições e as tornava transparentes aos olhos de um número cada vez maior de pessoas.
+(Modesto Florenzano. As revoluções burguesas, 1982. Adaptado.)
+Entre as críticas ao Antigo Regime, mencionadas no texto, podemos citar a rejeição iluminista ao</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>princípio da igualdade jurídica.</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>livre comércio.</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>liberalismo econômico.</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>republicanismo.</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>absolutismo monárquico.</t>
+        </is>
+      </c>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>Os filósofos iluministas teciam críticas ao Absolutismo monárquico pois esse feria o direito natural, ou seja, a afirmação de que todos eram iguais perante à lei e o exercício do poder baseado em explicações racionais.</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J627" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K627" t="inlineStr"/>
+      <c r="L627" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>O povo que possui o poder soberano deve fazer por si mesmo tudo o que pode fazer bem; e o que não puder fazer bem, deve fazê-lo por meio de seus ministros.
+Seus ministros não são seus se ele não os nomeia; logo, é uma máxima fundamental deste governo que o povo nomeie seus ministros, isto é, seus magistrados.
+MONTESQUIEU. O Espírito das Leis, Livro Segundo (adaptado). Disponível em:
+http://www.dhnet.org.br/direitos/anthist/marcos/hdh_montesquieu_o_espirito_das_leis.pdf. Acesso em 11 fev. 2020.
+A partir do excerto retirado de O Espírito das Leis, de Montesquieu, é correto afirmar que o pensamento iluminista</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>justificou pela religião o poder dos reis.</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>buscou conceber um sistema político justo.</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>promoveu ideias de sociedade sem Estado.</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>rejeitou toda forma de descentralização do poder.</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>defendeu a intervenção do Estado na economia.</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>Montesquieu, n'O Espírito das Leis, apresenta a necessidade de que o povo eleja magistrados para que assim, e somente assim, estes possam ter alguma autoridade sobre o povo. Os magistrados, os ministros, seriam do povo e teriam que se submeter aos seus desejos, algo que ia na contramão do sistema absolutista. Essas reflexões do movimento iluminista buscavam conceber um sistema baseado na justiça e na soberania do povo.</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K628" t="inlineStr"/>
+      <c r="L628" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>Resolvi fazer de conta que todas as coisas que até então haviam entrado no meu espírito não eram mais verdadeiras que as ilusões de meus sonhos. Mas, logo em seguida, adverti que, enquanto eu queria assim pensar que tudo era falso, cumpria necessariamente que eu, que pensava, fosse alguma coisa. E, notando que esta verdade: eu penso, logo existo, era tão firme e tão certa que todas as mais extravagantes suposições (...).
+DESCARTES, René. Discurso do Método, Parte IV.. São Paulo, LP&amp;M, 2005.
+A máxima de Descartes: eu penso, logo existo pode ser considerada parte das bases do pensamento Iluminista por</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>valorizar a centralidade do “eu” em oposição às filosofias renascentistas.</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>reafirmar a importância do autoconhecimento em oposição ao mundo externo.</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>refletir acerca da relevância dos sonhos na produção do conhecimento filosófico.</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>unir interpretações das perspectivas católica e renascentista em uma teoria.</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>destacar o valor da razão para se alcançar respostas justas e verdadeiras.</t>
+        </is>
+      </c>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>O Iluminismo é caracterizado pela valorização da verdade racional em oposição ao divino. Como é possível observar no excerto, o autor questiona-se acerca da veracidade dos elementos ao seu redor e sobre si mesmo. Sua existência, por sua vez, só pode ser confirmada pela certeza do uso de sua razão.</t>
+        </is>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K629" t="inlineStr"/>
+      <c r="L629" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>São verdades incontestáveis para nós: todos os homens nascem iguais; o Criador lhes conferiu certos direitos inalienáveis, entre os quais os de vida, o de liberdade e o de buscar a felicidade; para assegurar esses direitos se constituíram homens-governo cujos poderes justos emanam do consentimento dos governados; sempre que qualquer forma de governo tenda a destruir esses fins, assiste ao povo o direito de mudá-la ou aboli-la, instituindo um novo governo cujos princípios básicos e organização de poderes obedeçam às normas que lhes pareçam mais próprias para promover a segurança e a felicidade gerais.
+Trecho da Declaração de Independência dos Estados Unidos da América. Disponível em: https://www.uel.br/pessoal/jneto/gradua/historia/recdida/declaraindepeEUAHISJNeto.pdf. Acesso em: 01 nov. 2024.
+A Declaração de Independência dos EUA tem inspiração iluminista na medida em que</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>hierarquiza os homens a partir das famílias as quais pertencem e de sua riqueza.</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>define a supremacia plena dos governantes para fazer o que bem entenderem.</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>submete a autoridade dos governantes aos interesses das pessoas e não de um indivíduo.</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>justifica a liberdade dos homens como uma determinação divina definitiva.</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>determina que um governo justo está ligado aos interesses da Igreja.</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>O Iluminismo defende que o poder é emanado do povo, logo, o povo deveria escolher e legitimar seus governantes. Se os governantes não corresponderem às expectativas do povo, os governantes poderiam ser retirados do poder pelo povo. É precisamente essa ideia que é trabalhada no trecho da Declaração de Independência dos EUA.</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K630" t="inlineStr"/>
+      <c r="L630" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>Disponível em: https://upload.wikimedia.org/wikipedia/commons/7/7b/Index_Librorum_Prohibitorum_1.jpg. Acesso em: 01 nov. 2024.
+Em 1559, a Igreja Católica divulgou uma lista de livros proibidos por serem considerados opositores da fé, o Index. Diversos filósofos, escritores e cientistas tiveram suas obras incluídas no índice. Esse é um exemplo de que</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>a religião e a ciência coexistiram de forma pacífica durante a modernidade.</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>embora a ciência discordasse da religião em alguns aspectos, isso não era um impedimento de relacionamento pacífico pela perspectiva da religião.</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>embora a religião discordasse da ciência em alguns aspectos, isso não era um impedimento de relacionamento pacífico pela perspectiva da ciência.</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>ciência e religião tiveram uma relação conflituosa, incluindo casos de condenação de cientistas pela Santa Inquisição.</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>a religião e a ciência não coexistiram durante o mesmo período.</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>Com o avanço da ciência, temas defendidos pela Igreja passaram a ser contestados, como o geocentrismo, resultando, assim, na perseguição e no julgamento de pessoas acusadas de práticas heréticas, como os cientistas.</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J631" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="K631" t="inlineStr">
+        <is>
+          <t>8a_ph03_his_10.jpg</t>
+        </is>
+      </c>
+      <c r="L631" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>Naruto e Tartarugas Ninja fazem crossover em novo quadrinho da IDW
+Naruto e Tartarugas Ninja farão um crossover especial em nova edição de quadrinho da IDW, com lançamento em outubro nos EUA. As informações são do JBox.
+Foi divulgada uma primeira imagem do lançamento. No entanto, ressalta-se que ainda não se trata de uma versão final. Confira abaixo. 
+Disponível em: https://www.omelete.com.br/naruto/naruto-tartarugas-ninja-hq-crossover. Acesso em 11 de out de 2024.
+Qual o tipo de sujeito da frase em destaque no texto?</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Sujeito determinado composto.</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Sujeito determinado elíptico.</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Sujeito indeterminado.</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>Sujeito inexistente.</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>Sujeito simples.</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>Em "No entanto, ressalta-se que ainda não se trata de uma versão final", o pronome "se" indica que a ação do verbo não é atribuída a um sujeito específico, tornando o sujeito indeterminado. Dessa forma, não é possível identificar quem realiza a ação de "ressaltar", caracterizando o sujeito como indeterminado.</t>
+        </is>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J632" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K632" t="inlineStr"/>
+      <c r="L632" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>Nobel de Literatura: relembre os vencedores dos dez últimos anos
+Han Kang, escritora sul-coreana, ganhou o Prêmio Nobel de Literatura 2024. O anúncio foi feito nesta quinta-feira (10), pela Academia Sueca, em Estocolmo.
+De acordo com a academia, o prêmio foi concedido “por sua intensa prosa poética que confronta traumas históricos e expõe a fragilidade da vida humana".
+Disponível em: https://g1.globo.com/pop-arte/noticia/2024/10/10/nobel-de-literatura-relembre-os-vencedores-dos-ultimos-anos.ghtml. Acesso em 11 de out de 2024.
+Qual é o sujeito do segundo parágrafo da notícia?</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>"Fragilidade da vida humana".</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>"Traumas históricos".</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>"Prosa poética".</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>"Academia".</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>"Prêmio".</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>"Prêmio" é o sujeito da frase porque é o elemento que recebe a ação do verbo "foi concedido". Na frase, "o prêmio" é o que está sendo concedido pela academia, portanto, é o sujeito que realiza a ação principal da oração.</t>
+        </is>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J633" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K633" t="inlineStr"/>
+      <c r="L633" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>Taylor Swift doa US$ 5 milhões para ajudar vítimas dos furacões Milton e Helene nos Estados Unidos
+Informação foi anunciada pela Feeding America, organização sem fins lucrativos que constitui uma rede nacional de mais de 200 bancos alimentares.
+Taylor Swift doou US$ 5 milhões (aproximadamente R$ 27,9 milhões, na cotação atual) para ajudar as vítimas dos furacões Helene e Milton nos Estados Unidos. A informação foi anunciada pela Feeding America, organização sem fins lucrativos que constitui uma rede nacional de mais de 200 bancos alimentares.
+"Esta contribuição vai ajudar comunidades a reconstruir e se recuperar, provendo comida essencial, água limpa e suprimentos para pessoas afetadas por estas tempestades devastadoras. Juntos, podemos causar um impacto real ajudando famílias enquanto elas navegam os desafios à frente. Obrigado, Taylor, por se juntar a nós no movimento para acabar com a fome e ajudar comunidades necessitadas", escreveu a organização.
+Os EUA estão atravessando um período de fortes tempestades, com os furacões Helene e Milton. No final de setembro, o furacão Helene atingiu seis estados americanos, deixando ao menos 200 mortos.
+Já a noite da última quarta (9), o furacão Milton chegou ao estado da Flórida. O fenômeno foi considerado uma das tempestades mais poderosas que se formaram no Atlântico Norte nos últimos anos. A chegada do furacão deixou milhões de pessoas sem luz e provocou inundações na costa oeste do estado.
+Disponível em: Taylor Swift doa US$ 5 milhões para ajudar vítimas dos furacões Milton e Helene nos Estados Unidos | Pop &amp; Arte | G1 (globo.com). Acesso em: 11 out. 2024
+O texto acima se caracteriza como notícia e não como reportagem, pois</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>explora detalhadamente o contexto histórico dos furacões Helene e Milton.</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>inclui entrevistas com diversas fontes e perspectivas sobre a doação de Taylor Swift.</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>apresenta opiniões e análises sobre a importância das doações em situações de desastre.</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>fornece um relato breve e direto do evento, focando na doação de Taylor Swift e nas informações essenciais.</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>descreve minuciosamente os impactos econômicos que os furacões Helene e Milton causaram na vida da cantora Taylor Swift, que perdeu 5 milhões.</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>O texto fornece um relato breve e direto do evento, focando na doação de Taylor Swift e nas informações essenciais, como o valor da doação, a organização beneficiada e os impactos dos furacões. Isso caracteriza o texto como uma notícia. Se houvesse um aprofundamento maior nas informações, o texto se caracterizaria como reportagem.</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J634" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K634" t="inlineStr"/>
+      <c r="L634" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>Brasil supera a marca de 50 medalhas nos Jogos Paraolímpicos
+Nove novos pódios entre atletismo, natação e halterofilismo marcam o dia de competições na França. Em todas as conquistas brasileiras, a marca do Bolsa Atleta do Governo Federal
+Com mais quatro dias de competições ainda no horizonte dos Jogos Paralímpicos até o próximo domingo, a delegação brasileira já superou nesta quarta a marca de 50 medalhas em Paris. O feito simbólico veio com o bronze de Lara Lima na categoria até 41 quilos do halterofilismo.
+Ao longo do dia, o país subiu ao pódio outras oito vezes, entre atletismo e natação, com destaque para o sexto ouro de Maria Carolina Santiago, a brasileira com maior número de títulos na história dos Jogos. Carol venceu os 100m livre da classe S12 e fechou o revezamento 4 x 100m do Brasil que repetiu na França a prata de Tóquio.
+Ao todo, o Brasil soma 15 ouros, 15 pratas e 27 bronzes, um total de 57 medalhas, na sexta posição geral. A liderança permanece com a China, com 60 ouros e 131 medalhas.
+Até hoje, a melhor campanha do Brasil foi registrada em Tóquio, em 2021. No Japão, o Brasil somou 72 medalhas, com 22 ouros, 20 pratas e 30 bronzes. 
+Disponível em: Brasil supera a marca de 50 medalhas nos Jogos Paralímpicos — Secretaria de Comunicação Social (www.gov.br). Acesso em 14 de out. de 2024.
+Os dois últimos parágrafos destacados da notícia são classificados como</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>o terceiro parágrafo contém um período simples e o quarto parágrafo contém um período simples.</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>o terceiro parágrafo contém um período simples e o quarto parágrafo contém um período composto.</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>o terceiro parágrafo contém dois períodos simples e o quarto parágrafo contém dois períodos simples.</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>o terceiro parágrafo contém dois períodos simples e o quarto parágrafo contém um período composto.</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>o terceiro parágrafo contém um período composto e o quarto parágrafo contém dois períodos simples.</t>
+        </is>
+      </c>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>O terceiro parágrafo contém dois períodos simples, pois há apenas duas orações, isto é, uma frase que contenha um verbo (ou locução verbal). O mesmo acontece no quarto parágrafo, que contém dois períodos simples.</t>
+        </is>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J635" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K635" t="inlineStr"/>
+      <c r="L635" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>Leia a notícia a seguir.
+Por que gatos gostam mais dos homens que das mulheres? Estudo explica o motivo
+Pesquisa realizada em universidade da Turquia analisou 31 felinos domésticos e revelou uma possível seletividade comunicativa por parte dos animais
+Um dos principais achados foi a diferença de vocalização entre os gêneros dos tutores. Segundo os dados coletados, os gatos emitiram uma média de 4,3 miados ao reencontrar homens, enquanto vocalizaram 1,8 vezes diante de mulheres. A hipótese dos cientistas é que os felinos intensificam os sinais vocais com homens por perceberem menor frequência de interações verbais por parte desse grupo.
+[...]
+Apesar dos resultados, os pesquisadores alertam que o estudo tem limitações. A amostragem restrita e a condução do experimento exclusivamente na Turquia indicam a necessidade de novas investigações para determinar se os padrões observados se aplicam a gatos de outras culturas e ambientes. 
+Disponível em: https://exame.com/ciencia/por-que-gatos-gostam-mais-dos-homens-que-das-mulheres-estudo-explica-o-motivo/. Acesso em: 05 dez. 2025.
+Na notícia, identifica-se um sujeito determinado composto em</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>“Pesquisa realizada em universidade da Turquia analisou 31 felinos domésticos.”</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>“Apesar dos resultados, os pesquisadores alertam que o estudo tem limitações.”</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>“Um dos principais achados foi a diferença de vocalização entre os gêneros dos tutores.”</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>“[...] os felinos intensificam os sinais vocais com homens por perceberem menor frequência de interações verbais”</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>“A amostragem restrita e a condução do experimento exclusivamente na Turquia indicam a necessidade de novas investigações”</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>Na frase, o sujeito determinado composto é formado por "a amostragem restrita" e "a condução do experimento exclusivamente na Turquia". Ambos os elementos estão ligados pela conjunção "e", demonstrando que juntos realizam a ação de "indicar a necessidade de novas investigações". Assim, apresenta dois núcleos que compõem o sujeito da oração, caracterizando-o como um sujeito composto.</t>
+        </is>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K636" t="inlineStr"/>
+      <c r="L636" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>A princesa da água
+Ela era filha de um casal encantado, o rei do céu e a rainha da Terra. Ficou conhecida como a princesa das águas, porque tinha poderes sobre rios, riachos, cachoeiras… Era linda e sua beleza atraía muitos interessados em casar-se com ela. Mas foi o filho do Sol que conquistou seu coração. O casamento foi muito bonito e alegre, foram sete dias e sete noites de festividades.
+Quando a festa acabou, os noivos partiram para a casa do Sol. Chegando lá. a princesa das águas disse ao marido que pretendia passar com ele o ano inteiro, exceto três meses que havia de passar com sua mãe. Assim, todos os anos, a princesa das águas passava uma temporada com sua mãe debaixo do mar, num rico palácio de ouro e de brilhantes.
+O tempo correu e a princesa teve um filho. O principezinho ficava com o pai, quando a moça ia visitar sua mãe. Certo ano, porém, a princesa foi para a sua temporada com a mãe, como sempre, mas não a encontrou no palácio. A princesa perguntou sobre sua mãe aos peixes dos rios, às areias do mar, às conchas das praias, mas ninguém lhe respondia. Muito mais do que meses e anos se passaram nessa busca sem sucesso. Cansada e muito triste, ela retornou ao reino do Sol.
+Chegando lá, uma surpresa: o rei Sol havia se casado com outra e seu filho, já crescido, estava muito maltratado e triste. A princesa das águas, com muita raiva, pegou seu filho e se mudou para o fundo do mar. Deu ordem para que a maré subisse, e tudo ficou coberto pelas águas. No fundo do mar, a princesa e seu filho ficaram para sempre.
+Dizem que quem se atreve a olhar fixamente para a água do mar, vê a princesa, é encantado, cai na água e some para sempre.
+Disponível em: &lt;http://chc.org.br/artigo/a-princesa-da-agua/&gt;. Acesso em: 31 jan. 2020.
+Qual das sentenças retiradas do texto constitui um período simples?</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>“O tempo correu e a princesa teve um filho.”</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>“Quando a festa acabou, os noivos partiram para a casa do Sol.”</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>"O principezinho ficava com o pai, quando a moça ia visitar sua mãe."</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>“Era linda e sua beleza atraía muitos interessados em casar-se com ela.”</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>“Assim, todos os anos, a princesa das águas passava uma temporada com sua mãe debaixo do mar, num rico palácio de ouro e de brilhantes.”</t>
+        </is>
+      </c>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>Um período simples é aquele que contém apenas uma oração, sendo caracterizado pela presença de um único verbo ou locução verbal, que forma uma única oração. Na sentença "Assim, todos os anos, a princesa das águas passava uma temporada com sua mãe debaixo do mar, num rico palácio de ouro e de brilhantes.", o verbo "passava" é o único verbo presente, indicando uma única ação realizada pelo sujeito "a princesa das águas". Não há outras orações subordinadas ou coordenadas na frase, o que confirma que se trata de um período simples.</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K637" t="inlineStr">
+        <is>
+          <t>8a_ph03_por_06.png</t>
+        </is>
+      </c>
+      <c r="L637" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>Ela era filha de um casal encantado, o rei do céu e a rainha da Terra. Ficou conhecida como a princesa das águas, porque tinha poderes sobre rios, riachos, cachoeiras… Era linda e sua beleza atraía muitos interessados em casar-se com ela. Mas foi o filho do Sol que conquistou seu coração. O casamento foi muito bonito e alegre, foram sete dias e sete noites de festividades.
+Quando a festa acabou, os noivos partiram para a casa do Sol. Chegando lá, a princesa das águas disse ao marido que pretendia passar com ele o ano inteiro, exceto três meses que havia de passar com sua mãe. Assim, todos os anos, a princesa das águas passava uma temporada com sua mãe debaixo do mar, num rico palácio de ouro e de brilhantes.
+O tempo correu e a princesa teve um filho. O principezinho ficava com o pai, quando a moça ia visitar sua mãe. Certo ano, porém, a princesa foi para a sua temporada com a mãe, como sempre, mas não a encontrou no palácio. A princesa perguntou sobre sua mãe aos peixes dos rios, às areias do mar, às conchas das praias, mas ninguém lhe respondia. Muito mais do que meses e anos se passaram nessa busca sem sucesso. Cansada e muito triste, ela retornou ao reino do Sol.
+Chegando lá, uma surpresa: o rei Sol havia se casado com outra e seu filho, já crescido, estava muito maltratado e triste. A princesa das águas, com muita raiva, pegou seu filho e se mudou para o fundo do mar. Deu ordem para que a maré subisse, e tudo ficou coberto pelas águas. No fundo do mar, a princesa e seu filho ficaram para sempre. Dizem que quem se atreve a olhar fixamente para a água do mar, vê a princesa, é encantado, cai na água e some para sempre.
+Disponível em: &lt;http://chc.org.br/artigo/a-princesa-da-agua/&gt;. Acesso em: 31 jan. 2020
+Releia: “Ela era filha de um casal encantado, o rei do céu e a rainha da Terra.” Qual o sujeito do período?</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>“Ela”.</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>"Rei".</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>“Filha”.</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>“Casal”.</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>“Rainha”.</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>O sujeito é o termo da oração que indica quem ou o que realiza a ação expressa pelo verbo ou de quem ou do que se declara algo. No caso desta sentença, o verbo "era" está se referindo a "Ela", que é a pessoa sobre a qual se está fazendo uma declaração, informando que ela é filha de um casal encantado. As demais palavras na frase ("filha", "casal", "rei", "rainha") não desempenham o papel de sujeito, mas sim de complementos ou especificações adicionais dentro da oração. Portanto, "Ela" é o termo que exerce a função de sujeito.</t>
+        </is>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K638" t="inlineStr">
+        <is>
+          <t>8a_ph03_por_07.png</t>
+        </is>
+      </c>
+      <c r="L638" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>Ela era filha de um casal encantado, o rei do céu e a rainha da Terra. Ficou conhecida como a princesa das águas, porque tinha poderes sobre rios, riachos, cachoeiras… Era linda e sua beleza atraía muitos interessados em casar-se com ela. Mas foi o filho do Sol que conquistou seu coração. O casamento foi muito bonito e alegre, foram sete dias e sete noites de festividades.
+Quando a festa acabou, os noivos partiram para a casa do Sol. Chegando lá, a princesa das águas disse ao marido que pretendia passar com ele o ano inteiro, exceto três meses que havia de passar com sua mãe. Assim, todos os anos, a princesa das águas passava uma temporada com sua mãe debaixo do mar, num rico palácio de ouro e de brilhantes.
+O tempo correu e a princesa teve um filho. O principezinho ficava com o pai, quando a moça ia visitar sua mãe. Certo ano, porém, a princesa foi para a sua temporada com a mãe, como sempre, mas não a encontrou no palácio. A princesa perguntou sobre sua mãe aos peixes dos rios, às areias do mar, às conchas das praias, mas ninguém lhe respondia. Muito mais do que meses e anos se passaram nessa busca sem sucesso. Cansada e muito triste, ela retornou ao reino do Sol.
+Chegando lá, uma surpresa: o rei Sol havia se casado com outra e seu filho, já crescido, estava muito maltratado e triste. A princesa das águas, com muita raiva, pegou seu filho e se mudou para o fundo do mar. Deu ordem para que a maré subisse, e tudo ficou coberto pelas águas. No fundo do mar, a princesa e seu filho ficaram para sempre. Dizem que quem se atreve a olhar fixamente para a água do mar, vê a princesa, é encantado, cai na água e some para sempre.
+Disponível em: &lt;http://chc.org.br/artigo/a-princesa-da-agua/&gt;. Acesso em: 31 jan. 2020
+É exemplo de oração com sujeito desinencial:</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>"A princesa das águas, com muita raiva, pegou seu filho e se mudou para o fundo do mar."</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>“Muito mais do que meses e anos se passaram nessa busca sem sucesso.”</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>“Deu ordem para que a maré subisse, e tudo ficou coberto pelas águas.”</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>“Quando a festa acabou, os noivos partiram para a casa do Sol.”</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>“Cansada e muito triste, ela retornou ao reino do Sol.”</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>Uma oração com sujeito desinencial é aquela em que o sujeito não está explicitamente mencionado na frase, mas pode ser identificado pela desinência verbal, ou seja, pela terminação do verbo. Na sentença “Deu ordem para que a maré subisse, e tudo ficou coberto pelas águas.”, o verbo "deu" não tem um sujeito explícito na oração. No entanto, pelo contexto e pela conjugação do verbo, entende-se que o sujeito é "ele" ou "ela", que está implícito. Esse tipo de sujeito é chamado de desinencial ou elíptico porque não aparece na frase, mas pode ser inferido pelo leitor ou ouvinte. As demais alternativas apresentam sujeitos explícitos, ou seja, claramente mencionados na oração, o que não caracteriza um sujeito desinencial.</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K639" t="inlineStr">
+        <is>
+          <t>8a_ph03_por_08.png</t>
+        </is>
+      </c>
+      <c r="L639" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>Considere as sentenças a seguir:
+I. Rafael sempre foi um ótimo aluno.
+II. O caderno e os livros de Bruno ficaram em sua casa.
+III. Chegamos atrasadas para a aula de Literatura.
+IV. Choverá muito amanhã.
+V. Não avisaram qual será a sala de Thiago.
+Os sujeitos são classificados como:</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>I. Composto; II. Composto; III. Simples; IV. Inexistente; V. Oculto.</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>I. Composto; II. Simples; III. Oculto; IV. Indeterminado; V. Inexistente.</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>I. Simples; II. Composto; III. Oculto; IV. Inexistente; V. Indeterminado.</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>I. Simples; II. Composto; III. Inexistente; IV. Simples; V. Indeterminado.</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>I. Composto; II. Simples; III. Inexistente; IV. Indeterminado; V. Inexistente.</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>Na sentença I, "Rafael sempre foi um ótimo aluno", o sujeito é "Rafael", que é um sujeito simples por se tratar de um único núcleo.
+Na sentença II, "O caderno e os livros de Bruno ficaram em sua casa", o sujeito é "O caderno e os livros de Bruno", que é um sujeito composto por possuir dois núcleos ("caderno" e "livros").
+Na sentença III, "Chegamos atrasadas para a aula de Literatura", o sujeito é oculto, pois está implícito na forma verbal "chegamos", indicando "nós".
+Na sentença IV, "Choverá muito amanhã", o sujeito é inexistente, pois o verbo "chover" é impessoal e não se refere a nenhum sujeito.
+Na sentença V, "Não avisaram qual será a sala de Thiago", o sujeito é indeterminado, pois a forma verbal "avisaram" não especifica quem realizou a ação, podendo ser qualquer pessoa ou grupo.</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J640" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K640" t="inlineStr"/>
+      <c r="L640" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>É DESSA FLORESTA QUE SAI O CHAPEUZINHO VERMELHO,
+JOÃO E MARIA, OS IRMÃOS KARAMAZOV,
+A DAMA DAS CAMÉLIAS E OS TRÊS MOSQUETEIROS.
+Revista Bolsa, 1986. In: CARRASCOZA, J. A. A evolução do texto
+publicitário: a associação de palavras como elemento de sedução
+na publicidade. São Paulo: Futura, 1999 (adaptado).
+Sobre a sentença “É dessa floresta que sai o Chapeuzinho Vermelho, João e Maria, os Irmãos Karamazov, a Dama das CamélIas e Os Três Mosqueteiros.”, é possível afirmar que se trata de</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>um período composto.</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>uma frase não-verbal.</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>um período simples.</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>uma frase nominal.</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>uma oração sem sujeito.</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>"É dessa floresta que sai o Chapeuzinho Vermelho, João e Maria, os Irmãos Karamazov, a Dama das Camélias e Os Três Mosqueteiros." contém dois verbos: "é" e "sai". A presença desses dois verbos indica que a sentença é composta por duas orações: "É dessa floresta" e "que sai o Chapeuzinho Vermelho, João e Maria, os Irmãos Karamazov, a Dama das Camélias e Os Três Mosqueteiros." Quando uma sentença possui mais de uma oração, ela é classificada como um período composto.</t>
+        </is>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J641" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="K641" t="inlineStr">
+        <is>
+          <t>8a_ph03_por_10.jpg</t>
+        </is>
+      </c>
+      <c r="L641" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>Um grupo de amigos resolveu comprar ingressos para ir ao show de sua banda favorita. Eles compraram 4 ingressos e também pagaram uma taxa de serviço no valor de R$ 10,00.
+Qual das expressões a seguir calcula corretamente o valor gasto pelo grupo de amigos?</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_01_a.png]</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_01_b.png]</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_01_c.png]</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_01_d.png]</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_01_e.png]</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>A expressão correta é  pois eles compraram 4 ingressos a x reais cada e pagaram uma taxa de 10 reais.</t>
+        </is>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K642" t="inlineStr"/>
+      <c r="L642" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>Um grupo de amigos está organizando uma viagem de carro e calculou os custos totais da viagem, incluindo combustível, pedágios e alimentação. Eles expressaram o custo total da viagem na seguinte forma:
+onde y representa o custo por quilômetro rodado. Eles desejam simplificar essa expressão para entender melhor os custos totais da viagem.
+Qual é a expressão simplificada que o grupo deve usar?</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_02_a.png]</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_02_b.png]</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_02_c.png]</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_02_d.png]</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_02_e.png]</t>
+        </is>
+      </c>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>Simplificando a expressão, tem-se:</t>
+        </is>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K643" t="inlineStr">
+        <is>
+          <t>8a_ph03_mat_02.png</t>
+        </is>
+      </c>
+      <c r="L643" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>Um garoto está ajudando seu pai a planejar a reforma do quintal da casa. Ele precisa calcular a área do terreno que será coberto por grama. O terreno tem o formato de um retângulo, medindo 12 metros de comprimento por 4 metros de largura. No entanto, no centro desse terreno, há uma piscina retangular que mede 4 metros de comprimento por 3 metros de largura. Pedro precisa saber a área que será coberta por grama, excluindo a área da piscina.
+Qual é a área do terreno que será coberta por grama?</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_03_a.png]</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_03_b.png]</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_03_c.png]</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_03_d.png]</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_03_e.png]</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>A área total do terreno é calculada multiplicando o comprimento pela altura: 
+Logo, a área coberta por grama será:</t>
+        </is>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K644" t="inlineStr"/>
+      <c r="L644" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>Um grupo de amigos foi ao supermercado com R$ 150,00 e decidiu comprar produtos para o churrasco do fim de semana. Eles compraram dois pacotes de carne, cada um custando   reais, onde x é o peso em quilos, e um pacote de carvão que custa  reais, onde x também é o peso do carvão em Kg.
+Sabendo que o grupo gastou R$ 95,00 no total, qual foi o valor de x, que representa o peso dos produtos em kg?</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>8,75 kg</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>9,38 kg</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>15,63 kg</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>16,00 kg</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>27,00 kg</t>
+        </is>
+      </c>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>O custo total dos dois pacotes de carne e do pacote de carvão é dado por:
+Simplificando a expressão, tem-se que:</t>
+        </is>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K645" t="inlineStr">
+        <is>
+          <t>8a_ph03_mat_04.png</t>
+        </is>
+      </c>
+      <c r="L645" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>Um funcionário está construindo uma caixa em forma de bloco retangular para armazenar ferramentas. A caixa tem comprimento de  metros, largura de  metros e altura de x metros.
+Qual é a expressão algébrica que representa o volume da caixa?</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_05_a.png]</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_05_b.png]</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_05_c.png]</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_05_d.png]</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>[img:8a_ph03_mat_05_e.png]</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>volume de um bloco retangular é dado por  Portanto, a expressão algébrica para o volume da caixa é:
+Primeiro, multiplicamos (2x + 1) por (x - 2):
+Em seguida, multiplicamos o resultado por x:</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K646" t="inlineStr">
+        <is>
+          <t>8a_ph03_mat_05.png</t>
+        </is>
+      </c>
+      <c r="L646" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>Gabriel deseja comprar ladrilhos para sua casa, que está em construção. Como ele ainda não decidiu o tamanho da sua sala, mas sabe que ela terá o formato de um quadrado, ele pode então considerar que o lado medirá x metros.
+Se o preço dos ladrilhos é de 625 reais por metro quadrado, qual expressão algébrica representa o valor a ser pago, em reais, para ladrilhar sua sala?</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>25x</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>125x</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>125x²</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>625x</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>625x²</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>A área de sua sala será de x.x = x² metros quadrados. Como cada metro quadrado de ladrilho custa 625 reais, ele pagará 625x² reais.</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K647" t="inlineStr"/>
+      <c r="L647" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>Uma caixa d’água de 6 000 L está com a metade de sua capacidade preenchida. Uma bomba abastece a caixa d’água com 10 L de água por minuto.
+Qual é a expressão algébrica que representa a quantidade de água na caixa, considerando que passaram m minutos depois que a bomba foi ligada?</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>3 000 + 10m</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>3 000 + 100m</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>3 000 + 3 000m</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>6 000 + 10m</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>6 000 + 100m</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>Como a caixa já está cheia pela metade, há 3 000 L ocupados. Após m minutos, foram acrescentados 10m L na caixa.
+Logo, a expressão é 3 000 + 10m.</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K648" t="inlineStr"/>
+      <c r="L648" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>O pai de três filhas, Ana, Bianca e Carolina, deseja presenteá-las com chocolate pelo seu desempenho em matemática. Cada uma das filhas ganha de chocolate, em gramas, dez vezes a nota que tirar em matemática.
+Chamando a nota de Ana de A, a nota de Bianca de B e a nota de Carolina de C, qual expressão algébrica representa a quantidade de chocolate que o pai terá que comprar para presentear as filhas?</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>A + B + C</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>2A + 2B + 2C</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>10A + B + C</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>10A + B + 10C</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>10A + 10B + 10C</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>Ana receberá 10A gramas de chocolate, Bianca receberá 10B gramas de chocolate e Carolina receberá 10C gramas de chocolate.
+Portanto, o pai terá que comprar 10A + 10B + 10C gramas de chocolate.</t>
+        </is>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K649" t="inlineStr"/>
+      <c r="L649" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>João precisa pagar uma conta de 100 reais. Como ele sabe que não conseguirá pagar no dia, será cobrado uma multa por pagá-la atrasada. Ao ler o boleto da conta com mais detalhe, descobriu que a multa é de 2 reais para cada dia de atraso.
+Qual expressão algébrica representa o valor pago por João, considerando que houve um atraso de x dias?</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>102</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>100x</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>100 + x</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>100 + 2x</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>100 + 100x</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>João deve pagar um valor fixo de 100 reais mais x vezes a multa diária: 2x. Logo, a expressão é: 100 + 2x.</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K650" t="inlineStr"/>
+      <c r="L650" t="inlineStr">
+        <is>
+          <t>8ano</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>Em uma cidade, foi disponibilizado um sistema de aluguel de bicicletas que funciona da seguinte forma: paga-se uma mensalidade (valor fixo por mês) de R$ 25,00 e para cada hora andada com a bicicleta, paga-se R$ 2,50.
+Chamando de T o total pago no mês e h a quantidade de horas andadas de bicicleta, qual a expressão algébrica que representa a situação descrita?</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>T = 27,50</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>T = 25 + 2,50h</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>h = 25 + 2,50T</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>T = 25 + 25h</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>h = 25 + 25T</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>Há um valor fixo a ser pago: R$ 25,00. Além disso, será pago h vezes R$ 2,50 por hora de uso da bicicleta: 2,50h.
+Logo, a expressão será: T = 25 + 2,50h.</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>PH03</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="K651" t="inlineStr"/>
+      <c r="L651" t="inlineStr">
         <is>
           <t>8ano</t>
         </is>

</xml_diff>